<commit_message>
Close the Payday, Division 7A, benchmark and MCP findings from the September fact check
Closes the findings listed in the pull request from the 12 September 2026 fact check; the pull request records the verification.
</commit_message>
<xml_diff>
--- a/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
+++ b/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
@@ -6,7 +6,7 @@
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48B75D36-960B-4A31-A1DE-3E6D620BED93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E710A97-28BE-47D3-87D7-1AB664715363}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3510" yWindow="3510" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -690,10 +690,10 @@
     <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="out_of_scope_reason"/>
     <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="year_of_income_being_tested"/>
     <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Status">
-      <calculatedColumnFormula>IF(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),"SKIPPED",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&lt;1998,FALSE),"SKIPPED","REVIEWED"))</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","SKIPPED",IF(IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;1998,FALSE),"SKIPPED","REVIEWED"))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Floor_year">
-      <calculatedColumnFormula>IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),tblLoans[[#This Row],[year_loan_made]]&amp;"",tblLoans[[#This Row],[year_of_income_being_tested]]&amp;"")</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Floor_rate">
       <calculatedColumnFormula>IFERROR(INDEX(tblRates[rate],MATCH(tblLoans[[#This Row],[Floor_year]],tblRates[year_of_income],0)),"")</calculatedColumnFormula>
@@ -729,10 +729,10 @@
       <calculatedColumnFormula>IF(AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),ISNUMBER(Summary!$B$3),Summary!$B$3&gt;0,ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&gt;0),ROUND(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]*Summary!$B$3/(1-(1/(1+Summary!$B$3))^tblLoans[[#This Row],[Term_used]]),2),"")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="28" xr3:uid="{00000000-0010-0000-0000-00001C000000}" name="MYR_verdict">
-      <calculatedColumnFormula>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;""),tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")),TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")=Summary!$B$2,IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="29" xr3:uid="{00000000-0010-0000-0000-00001D000000}" name="MYR_reason">
-      <calculatedColumnFormula>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;"","gate benchmark year differs from year_loan_made",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),"gate benchmark year differs from year_loan_made",IF(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="30" xr3:uid="{00000000-0010-0000-0000-00001E000000}" name="MYR_required">
       <calculatedColumnFormula>IF(OR(tblLoans[[#This Row],[MYR_verdict]]="MYR_MET",tblLoans[[#This Row],[MYR_verdict]]="MYR_SHORT"),tblLoans[[#This Row],[MYR_raw]],"")</calculatedColumnFormula>
@@ -750,7 +750,7 @@
       <calculatedColumnFormula>IF(OR(_xlfn.ISFORMULA(tblLoans[[#This Row],[loan_id]]),_xlfn.ISFORMULA(tblLoans[[#This Row],[borrower_reference]]),_xlfn.ISFORMULA(tblLoans[[#This Row],[year_loan_made]]),_xlfn.ISFORMULA(tblLoans[[#This Row],[written_agreement]]),_xlfn.ISFORMULA(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]),_xlfn.ISFORMULA(tblLoans[[#This Row],[maximum_term_years]]),_xlfn.ISFORMULA(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]),_xlfn.ISFORMULA(tblLoans[[#This Row],[security_coverage_at_first_made]]),_xlfn.ISFORMULA(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),_xlfn.ISFORMULA(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),_xlfn.ISFORMULA(tblLoans[[#This Row],[remaining_term_years]]),_xlfn.ISFORMULA(tblLoans[[#This Row],[payments_applied_during_the_year]]),_xlfn.ISFORMULA(tblLoans[[#This Row],[out_of_scope_reason]]),_xlfn.ISFORMULA(tblLoans[[#This Row],[year_of_income_being_tested]])),1,0)</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="35" xr3:uid="{00000000-0010-0000-0000-000023000000}" name="Input_problem">
-      <calculatedColumnFormula>TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_loan_made]])=7,MID(tblLoans[[#This Row],[year_loan_made]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))+1,100)),FALSE))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_of_income_being_tested]])=7,MID(tblLoans[[#This Row],[year_of_income_being_tested]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))+1,100)),FALSE)))),"year label ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0))))),"number ",""))</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ABS(ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)-N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]))&gt;0.0000001,N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ABS(ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)-N(tblLoans[[#This Row],[payments_applied_during_the_year]]))&gt;0.0000001,N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="36" xr3:uid="{00000000-0010-0000-0000-000024000000}" name="Sample_row">
       <calculatedColumnFormula>IF(SUMPRODUCT((tblLoans[[#This Row],[loan_id]]&amp;""={"L-101","L-102","L-103","L-104","L-105","L-106","L-107","L-108"})*(tblLoans[[#This Row],[year_loan_made]]&amp;""={"2023-24","2022-23","2021-22","2024-25","2019-20","2020-21","2023-24","1996-97"}))&gt;0,1,0)</calculatedColumnFormula>
@@ -1300,11 +1300,11 @@
       <c r="M2" s="6"/>
       <c r="N2" s="6"/>
       <c r="O2" s="9" t="str">
-        <f>IF(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),"SKIPPED",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&lt;1998,FALSE),"SKIPPED","REVIEWED"))</f>
+        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","SKIPPED",IF(IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;1998,FALSE),"SKIPPED","REVIEWED"))</f>
         <v>REVIEWED</v>
       </c>
       <c r="P2" s="9" t="str">
-        <f>IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),tblLoans[[#This Row],[year_loan_made]]&amp;"",tblLoans[[#This Row],[year_of_income_being_tested]]&amp;"")</f>
+        <f>IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))</f>
         <v>2023-24</v>
       </c>
       <c r="Q2" s="9">
@@ -1352,11 +1352,11 @@
         <v>47212.37</v>
       </c>
       <c r="AB2" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;""),tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
+        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")),TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")=Summary!$B$2,IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
         <v>MYR_SHORT</v>
       </c>
       <c r="AC2" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;"","gate benchmark year differs from year_loan_made",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
+        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),"gate benchmark year differs from year_loan_made",IF(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
         <v/>
       </c>
       <c r="AD2" s="10">
@@ -1380,7 +1380,7 @@
         <v>0</v>
       </c>
       <c r="AI2" s="9" t="str">
-        <f>TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_loan_made]])=7,MID(tblLoans[[#This Row],[year_loan_made]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))+1,100)),FALSE))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_of_income_being_tested]])=7,MID(tblLoans[[#This Row],[year_of_income_being_tested]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))+1,100)),FALSE)))),"year label ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0))))),"number ",""))</f>
+        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ABS(ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)-N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]))&gt;0.0000001,N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ABS(ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)-N(tblLoans[[#This Row],[payments_applied_during_the_year]]))&gt;0.0000001,N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</f>
         <v/>
       </c>
       <c r="AJ2" s="9">
@@ -1428,11 +1428,11 @@
       <c r="M3" s="6"/>
       <c r="N3" s="6"/>
       <c r="O3" s="9" t="str">
-        <f>IF(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),"SKIPPED",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&lt;1998,FALSE),"SKIPPED","REVIEWED"))</f>
+        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","SKIPPED",IF(IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;1998,FALSE),"SKIPPED","REVIEWED"))</f>
         <v>REVIEWED</v>
       </c>
       <c r="P3" s="9" t="str">
-        <f>IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),tblLoans[[#This Row],[year_loan_made]]&amp;"",tblLoans[[#This Row],[year_of_income_being_tested]]&amp;"")</f>
+        <f>IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))</f>
         <v>2022-23</v>
       </c>
       <c r="Q3" s="9">
@@ -1480,11 +1480,11 @@
         <v>27640.06</v>
       </c>
       <c r="AB3" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;""),tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
+        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")),TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")=Summary!$B$2,IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
         <v>REFUSED</v>
       </c>
       <c r="AC3" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;"","gate benchmark year differs from year_loan_made",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
+        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),"gate benchmark year differs from year_loan_made",IF(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
         <v>s 109N gate is NOT_COMPLYING, so s 109E produces no repayment figure</v>
       </c>
       <c r="AD3" s="10" t="str">
@@ -1508,7 +1508,7 @@
         <v>0</v>
       </c>
       <c r="AI3" s="9" t="str">
-        <f>TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_loan_made]])=7,MID(tblLoans[[#This Row],[year_loan_made]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))+1,100)),FALSE))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_of_income_being_tested]])=7,MID(tblLoans[[#This Row],[year_of_income_being_tested]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))+1,100)),FALSE)))),"year label ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0))))),"number ",""))</f>
+        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ABS(ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)-N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]))&gt;0.0000001,N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ABS(ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)-N(tblLoans[[#This Row],[payments_applied_during_the_year]]))&gt;0.0000001,N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</f>
         <v/>
       </c>
       <c r="AJ3" s="9">
@@ -1556,11 +1556,11 @@
       <c r="M4" s="6"/>
       <c r="N4" s="6"/>
       <c r="O4" s="9" t="str">
-        <f>IF(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),"SKIPPED",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&lt;1998,FALSE),"SKIPPED","REVIEWED"))</f>
+        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","SKIPPED",IF(IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;1998,FALSE),"SKIPPED","REVIEWED"))</f>
         <v>REVIEWED</v>
       </c>
       <c r="P4" s="9" t="str">
-        <f>IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),tblLoans[[#This Row],[year_loan_made]]&amp;"",tblLoans[[#This Row],[year_of_income_being_tested]]&amp;"")</f>
+        <f>IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))</f>
         <v>2021-22</v>
       </c>
       <c r="Q4" s="9">
@@ -1608,11 +1608,11 @@
         <v>28334.799999999999</v>
       </c>
       <c r="AB4" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;""),tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
+        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")),TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")=Summary!$B$2,IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
         <v>REFUSED</v>
       </c>
       <c r="AC4" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;"","gate benchmark year differs from year_loan_made",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
+        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),"gate benchmark year differs from year_loan_made",IF(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
         <v>s 109N gate is UNKNOWN, so s 109E produces no repayment figure</v>
       </c>
       <c r="AD4" s="10" t="str">
@@ -1636,7 +1636,7 @@
         <v>0</v>
       </c>
       <c r="AI4" s="9" t="str">
-        <f>TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_loan_made]])=7,MID(tblLoans[[#This Row],[year_loan_made]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))+1,100)),FALSE))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_of_income_being_tested]])=7,MID(tblLoans[[#This Row],[year_of_income_being_tested]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))+1,100)),FALSE)))),"year label ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0))))),"number ",""))</f>
+        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ABS(ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)-N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]))&gt;0.0000001,N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ABS(ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)-N(tblLoans[[#This Row],[payments_applied_during_the_year]]))&gt;0.0000001,N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</f>
         <v/>
       </c>
       <c r="AJ4" s="9">
@@ -1684,11 +1684,11 @@
       <c r="M5" s="6"/>
       <c r="N5" s="6"/>
       <c r="O5" s="9" t="str">
-        <f>IF(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),"SKIPPED",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&lt;1998,FALSE),"SKIPPED","REVIEWED"))</f>
+        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","SKIPPED",IF(IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;1998,FALSE),"SKIPPED","REVIEWED"))</f>
         <v>REVIEWED</v>
       </c>
       <c r="P5" s="9" t="str">
-        <f>IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),tblLoans[[#This Row],[year_loan_made]]&amp;"",tblLoans[[#This Row],[year_of_income_being_tested]]&amp;"")</f>
+        <f>IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))</f>
         <v>2024-25</v>
       </c>
       <c r="Q5" s="9">
@@ -1736,11 +1736,11 @@
         <v>22489.279999999999</v>
       </c>
       <c r="AB5" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;""),tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
+        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")),TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")=Summary!$B$2,IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
         <v>UNKNOWN</v>
       </c>
       <c r="AC5" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;"","gate benchmark year differs from year_loan_made",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
+        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),"gate benchmark year differs from year_loan_made",IF(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
         <v>payments applied not established</v>
       </c>
       <c r="AD5" s="10" t="str">
@@ -1764,7 +1764,7 @@
         <v>0</v>
       </c>
       <c r="AI5" s="9" t="str">
-        <f>TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_loan_made]])=7,MID(tblLoans[[#This Row],[year_loan_made]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))+1,100)),FALSE))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_of_income_being_tested]])=7,MID(tblLoans[[#This Row],[year_of_income_being_tested]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))+1,100)),FALSE)))),"year label ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0))))),"number ",""))</f>
+        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ABS(ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)-N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]))&gt;0.0000001,N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ABS(ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)-N(tblLoans[[#This Row],[payments_applied_during_the_year]]))&gt;0.0000001,N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</f>
         <v/>
       </c>
       <c r="AJ5" s="9">
@@ -1812,11 +1812,11 @@
       <c r="M6" s="6"/>
       <c r="N6" s="6"/>
       <c r="O6" s="9" t="str">
-        <f>IF(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),"SKIPPED",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&lt;1998,FALSE),"SKIPPED","REVIEWED"))</f>
+        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","SKIPPED",IF(IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;1998,FALSE),"SKIPPED","REVIEWED"))</f>
         <v>REVIEWED</v>
       </c>
       <c r="P6" s="9" t="str">
-        <f>IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),tblLoans[[#This Row],[year_loan_made]]&amp;"",tblLoans[[#This Row],[year_of_income_being_tested]]&amp;"")</f>
+        <f>IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))</f>
         <v>2019-20</v>
       </c>
       <c r="Q6" s="9">
@@ -1864,11 +1864,11 @@
         <v/>
       </c>
       <c r="AB6" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;""),tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
+        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")),TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")=Summary!$B$2,IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
         <v>REFUSED</v>
       </c>
       <c r="AC6" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;"","gate benchmark year differs from year_loan_made",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
+        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),"gate benchmark year differs from year_loan_made",IF(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
         <v>nil remaining term under s 109E(6)</v>
       </c>
       <c r="AD6" s="10" t="str">
@@ -1892,7 +1892,7 @@
         <v>0</v>
       </c>
       <c r="AI6" s="9" t="str">
-        <f>TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_loan_made]])=7,MID(tblLoans[[#This Row],[year_loan_made]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))+1,100)),FALSE))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_of_income_being_tested]])=7,MID(tblLoans[[#This Row],[year_of_income_being_tested]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))+1,100)),FALSE)))),"year label ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0))))),"number ",""))</f>
+        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ABS(ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)-N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]))&gt;0.0000001,N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ABS(ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)-N(tblLoans[[#This Row],[payments_applied_during_the_year]]))&gt;0.0000001,N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</f>
         <v/>
       </c>
       <c r="AJ6" s="9">
@@ -1940,11 +1940,11 @@
       <c r="M7" s="6"/>
       <c r="N7" s="6"/>
       <c r="O7" s="9" t="str">
-        <f>IF(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),"SKIPPED",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&lt;1998,FALSE),"SKIPPED","REVIEWED"))</f>
+        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","SKIPPED",IF(IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;1998,FALSE),"SKIPPED","REVIEWED"))</f>
         <v>REVIEWED</v>
       </c>
       <c r="P7" s="9" t="str">
-        <f>IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),tblLoans[[#This Row],[year_loan_made]]&amp;"",tblLoans[[#This Row],[year_of_income_being_tested]]&amp;"")</f>
+        <f>IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))</f>
         <v>2020-21</v>
       </c>
       <c r="Q7" s="9">
@@ -1992,11 +1992,11 @@
         <v>36713.81</v>
       </c>
       <c r="AB7" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;""),tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
+        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")),TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")=Summary!$B$2,IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
         <v>REFUSED</v>
       </c>
       <c r="AC7" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;"","gate benchmark year differs from year_loan_made",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
+        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),"gate benchmark year differs from year_loan_made",IF(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
         <v>s 109N gate is NOT_COMPLYING, so s 109E produces no repayment figure</v>
       </c>
       <c r="AD7" s="10" t="str">
@@ -2020,7 +2020,7 @@
         <v>0</v>
       </c>
       <c r="AI7" s="9" t="str">
-        <f>TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_loan_made]])=7,MID(tblLoans[[#This Row],[year_loan_made]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))+1,100)),FALSE))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_of_income_being_tested]])=7,MID(tblLoans[[#This Row],[year_of_income_being_tested]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))+1,100)),FALSE)))),"year label ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0))))),"number ",""))</f>
+        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ABS(ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)-N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]))&gt;0.0000001,N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ABS(ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)-N(tblLoans[[#This Row],[payments_applied_during_the_year]]))&gt;0.0000001,N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</f>
         <v/>
       </c>
       <c r="AJ7" s="9">
@@ -2070,11 +2070,11 @@
       </c>
       <c r="N8" s="6"/>
       <c r="O8" s="9" t="str">
-        <f>IF(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),"SKIPPED",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&lt;1998,FALSE),"SKIPPED","REVIEWED"))</f>
+        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","SKIPPED",IF(IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;1998,FALSE),"SKIPPED","REVIEWED"))</f>
         <v>SKIPPED</v>
       </c>
       <c r="P8" s="9" t="str">
-        <f>IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),tblLoans[[#This Row],[year_loan_made]]&amp;"",tblLoans[[#This Row],[year_of_income_being_tested]]&amp;"")</f>
+        <f>IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))</f>
         <v>2023-24</v>
       </c>
       <c r="Q8" s="9">
@@ -2122,11 +2122,11 @@
         <v/>
       </c>
       <c r="AB8" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;""),tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
+        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")),TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")=Summary!$B$2,IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
         <v/>
       </c>
       <c r="AC8" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;"","gate benchmark year differs from year_loan_made",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
+        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),"gate benchmark year differs from year_loan_made",IF(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
         <v/>
       </c>
       <c r="AD8" s="10" t="str">
@@ -2150,7 +2150,7 @@
         <v>0</v>
       </c>
       <c r="AI8" s="9" t="str">
-        <f>TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_loan_made]])=7,MID(tblLoans[[#This Row],[year_loan_made]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))+1,100)),FALSE))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_of_income_being_tested]])=7,MID(tblLoans[[#This Row],[year_of_income_being_tested]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))+1,100)),FALSE)))),"year label ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0))))),"number ",""))</f>
+        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ABS(ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)-N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]))&gt;0.0000001,N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ABS(ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)-N(tblLoans[[#This Row],[payments_applied_during_the_year]]))&gt;0.0000001,N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</f>
         <v/>
       </c>
       <c r="AJ8" s="9">
@@ -2198,11 +2198,11 @@
       <c r="M9" s="6"/>
       <c r="N9" s="6"/>
       <c r="O9" s="9" t="str">
-        <f>IF(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),"SKIPPED",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&lt;1998,FALSE),"SKIPPED","REVIEWED"))</f>
+        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","SKIPPED",IF(IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;1998,FALSE),"SKIPPED","REVIEWED"))</f>
         <v>SKIPPED</v>
       </c>
       <c r="P9" s="9" t="str">
-        <f>IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),tblLoans[[#This Row],[year_loan_made]]&amp;"",tblLoans[[#This Row],[year_of_income_being_tested]]&amp;"")</f>
+        <f>IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))</f>
         <v>1996-97</v>
       </c>
       <c r="Q9" s="9" t="str">
@@ -2250,11 +2250,11 @@
         <v/>
       </c>
       <c r="AB9" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;""),tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
+        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")),TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")=Summary!$B$2,IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
         <v/>
       </c>
       <c r="AC9" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[year_loan_made]]&amp;"","gate benchmark year differs from year_loan_made",IF(tblLoans[[#This Row],[year_loan_made]]&amp;""=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
+        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),"gate benchmark year differs from year_loan_made",IF(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
         <v/>
       </c>
       <c r="AD9" s="10" t="str">
@@ -2278,7 +2278,7 @@
         <v>0</v>
       </c>
       <c r="AI9" s="9" t="str">
-        <f>TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_loan_made]])=7,MID(tblLoans[[#This Row],[year_loan_made]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))+1,100)),FALSE))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_of_income_being_tested]])=7,MID(tblLoans[[#This Row],[year_of_income_being_tested]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))+1,100)),FALSE)))),"year label ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0))))),"number ",""))</f>
+        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ABS(ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)-N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]))&gt;0.0000001,N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ABS(ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)-N(tblLoans[[#This Row],[payments_applied_during_the_year]]))&gt;0.0000001,N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</f>
         <v/>
       </c>
       <c r="AJ9" s="9">

</xml_diff>

<commit_message>
Test the exact cent figure, bound the Summary coverage date and retry busy COM calls in the Payday builder
Review follow-ups: the Division 7A money guard uses ROUND(x,2)<>x so a third decimal place is refused as parse_money refuses it; the Payday coverage date is held to the same sane-date bound as the as-at date; the MCP instructions continue only while a next_offset is returned; the Payday builder retries a null Open and RPC_E_CALL_REJECTED. Both workbooks rebuilt through Excel 16.0 build 20430.
</commit_message>
<xml_diff>
--- a/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
+++ b/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
@@ -6,7 +6,7 @@
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E710A97-28BE-47D3-87D7-1AB664715363}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AD8E472-22D5-4F8F-BA8B-5147CC4BEA3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3510" yWindow="3510" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -750,7 +750,7 @@
       <calculatedColumnFormula>IF(OR(_xlfn.ISFORMULA(tblLoans[[#This Row],[loan_id]]),_xlfn.ISFORMULA(tblLoans[[#This Row],[borrower_reference]]),_xlfn.ISFORMULA(tblLoans[[#This Row],[year_loan_made]]),_xlfn.ISFORMULA(tblLoans[[#This Row],[written_agreement]]),_xlfn.ISFORMULA(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]),_xlfn.ISFORMULA(tblLoans[[#This Row],[maximum_term_years]]),_xlfn.ISFORMULA(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]),_xlfn.ISFORMULA(tblLoans[[#This Row],[security_coverage_at_first_made]]),_xlfn.ISFORMULA(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),_xlfn.ISFORMULA(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),_xlfn.ISFORMULA(tblLoans[[#This Row],[remaining_term_years]]),_xlfn.ISFORMULA(tblLoans[[#This Row],[payments_applied_during_the_year]]),_xlfn.ISFORMULA(tblLoans[[#This Row],[out_of_scope_reason]]),_xlfn.ISFORMULA(tblLoans[[#This Row],[year_of_income_being_tested]])),1,0)</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="35" xr3:uid="{00000000-0010-0000-0000-000023000000}" name="Input_problem">
-      <calculatedColumnFormula>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ABS(ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)-N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]))&gt;0.0000001,N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ABS(ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)-N(tblLoans[[#This Row],[payments_applied_during_the_year]]))&gt;0.0000001,N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[payments_applied_during_the_year]]),N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="36" xr3:uid="{00000000-0010-0000-0000-000024000000}" name="Sample_row">
       <calculatedColumnFormula>IF(SUMPRODUCT((tblLoans[[#This Row],[loan_id]]&amp;""={"L-101","L-102","L-103","L-104","L-105","L-106","L-107","L-108"})*(tblLoans[[#This Row],[year_loan_made]]&amp;""={"2023-24","2022-23","2021-22","2024-25","2019-20","2020-21","2023-24","1996-97"}))&gt;0,1,0)</calculatedColumnFormula>
@@ -1380,7 +1380,7 @@
         <v>0</v>
       </c>
       <c r="AI2" s="9" t="str">
-        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ABS(ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)-N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]))&gt;0.0000001,N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ABS(ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)-N(tblLoans[[#This Row],[payments_applied_during_the_year]]))&gt;0.0000001,N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</f>
+        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[payments_applied_during_the_year]]),N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</f>
         <v/>
       </c>
       <c r="AJ2" s="9">
@@ -1508,7 +1508,7 @@
         <v>0</v>
       </c>
       <c r="AI3" s="9" t="str">
-        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ABS(ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)-N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]))&gt;0.0000001,N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ABS(ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)-N(tblLoans[[#This Row],[payments_applied_during_the_year]]))&gt;0.0000001,N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</f>
+        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[payments_applied_during_the_year]]),N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</f>
         <v/>
       </c>
       <c r="AJ3" s="9">
@@ -1636,7 +1636,7 @@
         <v>0</v>
       </c>
       <c r="AI4" s="9" t="str">
-        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ABS(ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)-N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]))&gt;0.0000001,N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ABS(ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)-N(tblLoans[[#This Row],[payments_applied_during_the_year]]))&gt;0.0000001,N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</f>
+        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[payments_applied_during_the_year]]),N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</f>
         <v/>
       </c>
       <c r="AJ4" s="9">
@@ -1764,7 +1764,7 @@
         <v>0</v>
       </c>
       <c r="AI5" s="9" t="str">
-        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ABS(ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)-N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]))&gt;0.0000001,N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ABS(ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)-N(tblLoans[[#This Row],[payments_applied_during_the_year]]))&gt;0.0000001,N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</f>
+        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[payments_applied_during_the_year]]),N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</f>
         <v/>
       </c>
       <c r="AJ5" s="9">
@@ -1892,7 +1892,7 @@
         <v>0</v>
       </c>
       <c r="AI6" s="9" t="str">
-        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ABS(ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)-N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]))&gt;0.0000001,N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ABS(ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)-N(tblLoans[[#This Row],[payments_applied_during_the_year]]))&gt;0.0000001,N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</f>
+        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[payments_applied_during_the_year]]),N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</f>
         <v/>
       </c>
       <c r="AJ6" s="9">
@@ -2020,7 +2020,7 @@
         <v>0</v>
       </c>
       <c r="AI7" s="9" t="str">
-        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ABS(ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)-N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]))&gt;0.0000001,N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ABS(ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)-N(tblLoans[[#This Row],[payments_applied_during_the_year]]))&gt;0.0000001,N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</f>
+        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[payments_applied_during_the_year]]),N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</f>
         <v/>
       </c>
       <c r="AJ7" s="9">
@@ -2150,7 +2150,7 @@
         <v>0</v>
       </c>
       <c r="AI8" s="9" t="str">
-        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ABS(ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)-N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]))&gt;0.0000001,N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ABS(ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)-N(tblLoans[[#This Row],[payments_applied_during_the_year]]))&gt;0.0000001,N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</f>
+        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[payments_applied_during_the_year]]),N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</f>
         <v/>
       </c>
       <c r="AJ8" s="9">
@@ -2278,7 +2278,7 @@
         <v>0</v>
       </c>
       <c r="AI9" s="9" t="str">
-        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ABS(ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)-N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]))&gt;0.0000001,N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ABS(ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)-N(tblLoans[[#This Row],[payments_applied_during_the_year]]))&gt;0.0000001,N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</f>
+        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[payments_applied_during_the_year]]),N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</f>
         <v/>
       </c>
       <c r="AJ9" s="9">

</xml_diff>

<commit_message>
Correct workbook rates, validation and Division 7A caveats
</commit_message>
<xml_diff>
--- a/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
+++ b/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
@@ -6,7 +6,7 @@
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AD8E472-22D5-4F8F-BA8B-5147CC4BEA3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA084D99-9AAC-4EBC-B672-6DE10659BCA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3510" yWindow="3510" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -401,7 +401,7 @@
     <t>No formula in an input cell</t>
   </si>
   <si>
-    <t>A reviewed benchmark rate exists for the year of income</t>
+    <t>A reviewed benchmark exists and every table rate is a number from zero to one</t>
   </si>
   <si>
     <t>Every reviewed loan is on s 109N terms</t>
@@ -422,7 +422,7 @@
     <t>Caveats the engine attaches to every result</t>
   </si>
   <si>
-    <t>COMPLYING means the four limbs of s 109N(1) are established on the operator's own facts. The lodgment day (s 109D(6)) is asserted, not computed. Refinancing reductions to the maximum term (s 109N(3A) to (3D)) and the other Subdivision D exclusions are not modelled.</t>
+    <t>Interest-floor interpretation unresolved: ATO guidance requires the benchmark interest rate for each year of the loan. This workbook compares one selected year's benchmark and defaults to the year the loan was made. COMPLYING does not establish that the agreement meets the annual interest requirement. Review the agreement and relevant years before relying on this result. See docs/primary-source-review-2026-08-31.md. The lodgment day (s 109D(6)) is asserted, not computed. Refinancing reductions to the maximum term (s 109N(3A) to (3D)) and the other Subdivision D exclusions are not modelled.</t>
   </si>
   <si>
     <t>s 109R: the workbook does not decide whether the payments applied are genuine repayments. The figure used is the operator's assertion.</t>
@@ -2756,7 +2756,7 @@
         <v>121</v>
       </c>
       <c r="B4" s="9" t="str">
-        <f>IF(ISNUMBER(Summary!B3),"PASS","BLOCKED")</f>
+        <f>IFERROR(IF(AND(ISNUMBER(Summary!B3),COUNT(tblRates[rate])=ROWS(tblRates[rate]),MIN(tblRates[rate])&gt;=0,MAX(tblRates[rate])&lt;=1),"PASS","BLOCKED"),"BLOCKED")</f>
         <v>PASS</v>
       </c>
       <c r="C4" s="9" t="str">
@@ -2864,7 +2864,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" ht="135" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
         <v>128</v>
       </c>

</xml_diff>

<commit_message>
Correct workbook rates, validation and Division 7A caveats (#171)
Add the published October-December 2026 GIC rate and reject invalid workbook rate overrides. Expose the unresolved annual Division 7A interest-floor interpretation in the engine, workbook and MCP demonstration. Include the workbook builder in source archives and correct two release-verification signer references.
</commit_message>
<xml_diff>
--- a/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
+++ b/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
@@ -6,7 +6,7 @@
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AD8E472-22D5-4F8F-BA8B-5147CC4BEA3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA084D99-9AAC-4EBC-B672-6DE10659BCA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3510" yWindow="3510" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -401,7 +401,7 @@
     <t>No formula in an input cell</t>
   </si>
   <si>
-    <t>A reviewed benchmark rate exists for the year of income</t>
+    <t>A reviewed benchmark exists and every table rate is a number from zero to one</t>
   </si>
   <si>
     <t>Every reviewed loan is on s 109N terms</t>
@@ -422,7 +422,7 @@
     <t>Caveats the engine attaches to every result</t>
   </si>
   <si>
-    <t>COMPLYING means the four limbs of s 109N(1) are established on the operator's own facts. The lodgment day (s 109D(6)) is asserted, not computed. Refinancing reductions to the maximum term (s 109N(3A) to (3D)) and the other Subdivision D exclusions are not modelled.</t>
+    <t>Interest-floor interpretation unresolved: ATO guidance requires the benchmark interest rate for each year of the loan. This workbook compares one selected year's benchmark and defaults to the year the loan was made. COMPLYING does not establish that the agreement meets the annual interest requirement. Review the agreement and relevant years before relying on this result. See docs/primary-source-review-2026-08-31.md. The lodgment day (s 109D(6)) is asserted, not computed. Refinancing reductions to the maximum term (s 109N(3A) to (3D)) and the other Subdivision D exclusions are not modelled.</t>
   </si>
   <si>
     <t>s 109R: the workbook does not decide whether the payments applied are genuine repayments. The figure used is the operator's assertion.</t>
@@ -2756,7 +2756,7 @@
         <v>121</v>
       </c>
       <c r="B4" s="9" t="str">
-        <f>IF(ISNUMBER(Summary!B3),"PASS","BLOCKED")</f>
+        <f>IFERROR(IF(AND(ISNUMBER(Summary!B3),COUNT(tblRates[rate])=ROWS(tblRates[rate]),MIN(tblRates[rate])&gt;=0,MAX(tblRates[rate])&lt;=1),"PASS","BLOCKED"),"BLOCKED")</f>
         <v>PASS</v>
       </c>
       <c r="C4" s="9" t="str">
@@ -2864,7 +2864,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" ht="135" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
         <v>128</v>
       </c>

</xml_diff>

<commit_message>
fix: block duplicate Division 7A benchmark years
</commit_message>
<xml_diff>
--- a/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
+++ b/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
@@ -6,7 +6,7 @@
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA084D99-9AAC-4EBC-B672-6DE10659BCA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{235D3489-AEE8-4029-9C94-487CEFEC45FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3510" yWindow="3510" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -401,7 +401,7 @@
     <t>No formula in an input cell</t>
   </si>
   <si>
-    <t>A reviewed benchmark exists and every table rate is a number from zero to one</t>
+    <t>A reviewed benchmark exists, rate years are unique and rates are from zero to one</t>
   </si>
   <si>
     <t>Every reviewed loan is on s 109N terms</t>
@@ -2756,7 +2756,7 @@
         <v>121</v>
       </c>
       <c r="B4" s="9" t="str">
-        <f>IFERROR(IF(AND(ISNUMBER(Summary!B3),COUNT(tblRates[rate])=ROWS(tblRates[rate]),MIN(tblRates[rate])&gt;=0,MAX(tblRates[rate])&lt;=1),"PASS","BLOCKED"),"BLOCKED")</f>
+        <f>IFERROR(IF(AND(ISNUMBER(Summary!B3),COUNT(tblRates[rate])=ROWS(tblRates[rate]),SUMPRODUCT(--(COUNTIF(tblRates[year_of_income],tblRates[year_of_income])&lt;&gt;1))=0,MIN(tblRates[rate])&gt;=0,MAX(tblRates[rate])&lt;=1),"PASS","BLOCKED"),"BLOCKED")</f>
         <v>PASS</v>
       </c>
       <c r="C4" s="9" t="str">

</xml_diff>

<commit_message>
fix: block duplicate Division 7A benchmark years (#175)
Duplicate benchmark-year labels could silently select the first rate. The workbook now blocks duplicate years, including duplicates whose rates agree (F034). Loan calculations and source rates are unchanged.

Verification: 326 tests passed, 6 skipped, 95% coverage; Ruff, mypy, dependency audit and build passed. Native Excel accepts unique years and blocks both duplicate controls. Only the check label and formula changed; other cells and styles match the baseline.
</commit_message>
<xml_diff>
--- a/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
+++ b/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
@@ -6,7 +6,7 @@
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA084D99-9AAC-4EBC-B672-6DE10659BCA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{235D3489-AEE8-4029-9C94-487CEFEC45FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3510" yWindow="3510" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -401,7 +401,7 @@
     <t>No formula in an input cell</t>
   </si>
   <si>
-    <t>A reviewed benchmark exists and every table rate is a number from zero to one</t>
+    <t>A reviewed benchmark exists, rate years are unique and rates are from zero to one</t>
   </si>
   <si>
     <t>Every reviewed loan is on s 109N terms</t>
@@ -2756,7 +2756,7 @@
         <v>121</v>
       </c>
       <c r="B4" s="9" t="str">
-        <f>IFERROR(IF(AND(ISNUMBER(Summary!B3),COUNT(tblRates[rate])=ROWS(tblRates[rate]),MIN(tblRates[rate])&gt;=0,MAX(tblRates[rate])&lt;=1),"PASS","BLOCKED"),"BLOCKED")</f>
+        <f>IFERROR(IF(AND(ISNUMBER(Summary!B3),COUNT(tblRates[rate])=ROWS(tblRates[rate]),SUMPRODUCT(--(COUNTIF(tblRates[year_of_income],tblRates[year_of_income])&lt;&gt;1))=0,MIN(tblRates[rate])&gt;=0,MAX(tblRates[rate])&lt;=1),"PASS","BLOCKED"),"BLOCKED")</f>
         <v>PASS</v>
       </c>
       <c r="C4" s="9" t="str">

</xml_diff>

<commit_message>
Prepare div7a-loan-review 0.1.3 and pin the MCP server to it
The MCP adapters on main read the rate-table manifest that
div7a-loan-review gained in #182, which is unreleased. Against
published 0.1.2 the MCP suite fails 40 Division 7A tests, so 0.2.3
cannot ship until the engine does. Bump the engine to 0.1.3 with its
release note, rebuild the workbook through Excel, regenerate its
standalone lock, pin the MCP server to 0.1.3 and regenerate the checked
demo transcript. The MCP standalone lock follows once PyPI holds 0.1.3.
</commit_message>
<xml_diff>
--- a/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
+++ b/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
@@ -6,9 +6,9 @@
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{235D3489-AEE8-4029-9C94-487CEFEC45FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB0F81A0-04EF-404E-8CD4-A4F65CFA007C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3510" yWindow="3510" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="38700" windowHeight="15885" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Start Here" sheetId="1" r:id="rId1"/>
@@ -62,7 +62,7 @@
     <t>Overall status</t>
   </si>
   <si>
-    <t>div7a-loan-review workbook, engine 0.1.2. Macro-free. Not advice; see DISCLAIMER.md in the repository.</t>
+    <t>div7a-loan-review workbook, engine 0.1.3. Macro-free. Not advice; see DISCLAIMER.md in the repository.</t>
   </si>
   <si>
     <t>loan_id</t>
@@ -446,7 +446,7 @@
     <t>Workbook engine version</t>
   </si>
   <si>
-    <t>0.1.2</t>
+    <t>0.1.3</t>
   </si>
   <si>
     <t>Desktop Excel build used to calculate cached values</t>

</xml_diff>

<commit_message>
Prepare div7a-loan-review 0.1.4 and pin the MCP server to it
Bump div7a-loan-review to 0.1.4 so the unreleased RBA primary-source
provenance from #213 reaches PyPI, and move the MCP server's pin to it.

No engine logic changes: div7aloan/__init__.py carries only the version
string, and no benchmark rate value moves.
</commit_message>
<xml_diff>
--- a/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
+++ b/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
@@ -6,7 +6,7 @@
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB0F81A0-04EF-404E-8CD4-A4F65CFA007C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00DAA400-1921-4237-86A9-527DE9E5DEA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1560" yWindow="1560" windowWidth="38700" windowHeight="15885" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -62,7 +62,7 @@
     <t>Overall status</t>
   </si>
   <si>
-    <t>div7a-loan-review workbook, engine 0.1.3. Macro-free. Not advice; see DISCLAIMER.md in the repository.</t>
+    <t>div7a-loan-review workbook, engine 0.1.4. Macro-free. Not advice; see DISCLAIMER.md in the repository.</t>
   </si>
   <si>
     <t>loan_id</t>
@@ -446,7 +446,7 @@
     <t>Workbook engine version</t>
   </si>
   <si>
-    <t>0.1.3</t>
+    <t>0.1.4</t>
   </si>
   <si>
     <t>Desktop Excel build used to calculate cached values</t>

</xml_diff>

<commit_message>
Prepare div7a-loan-review 0.1.4 and pin the MCP server to it (#228)
Bump div7a-loan-review to 0.1.4 so the unreleased RBA primary-source
provenance from #213 reaches PyPI, and move the MCP server's pin to it.

No engine logic changes: div7aloan/__init__.py carries only the version
string, and no benchmark rate value moves. The MCP standalone uv.lock is
regenerated in a follow-up once PyPI holds 0.1.4.
</commit_message>
<xml_diff>
--- a/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
+++ b/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
@@ -6,7 +6,7 @@
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB0F81A0-04EF-404E-8CD4-A4F65CFA007C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00DAA400-1921-4237-86A9-527DE9E5DEA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1560" yWindow="1560" windowWidth="38700" windowHeight="15885" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -62,7 +62,7 @@
     <t>Overall status</t>
   </si>
   <si>
-    <t>div7a-loan-review workbook, engine 0.1.3. Macro-free. Not advice; see DISCLAIMER.md in the repository.</t>
+    <t>div7a-loan-review workbook, engine 0.1.4. Macro-free. Not advice; see DISCLAIMER.md in the repository.</t>
   </si>
   <si>
     <t>loan_id</t>
@@ -446,7 +446,7 @@
     <t>Workbook engine version</t>
   </si>
   <si>
-    <t>0.1.3</t>
+    <t>0.1.4</t>
   </si>
   <si>
     <t>Desktop Excel build used to calculate cached values</t>

</xml_diff>

<commit_message>
Rebuild the Div 7A workbook with the RateYears selector
Built by tools/build_workbook.py through desktop Excel on top of current main, so the Summary year selector's defined name and main's later workbook changes are in one file. tools/check_workbook_rate_years.ps1 passes all three cases.
</commit_message>
<xml_diff>
--- a/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
+++ b/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
@@ -6,9 +6,9 @@
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00DAA400-1921-4237-86A9-527DE9E5DEA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B9C2A8D-EFF4-4CA2-B3A4-A1B9462A8FCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="1560" windowWidth="38700" windowHeight="15885" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="390" yWindow="390" windowWidth="38700" windowHeight="15885" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Start Here" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,9 @@
     <sheet name="Review Checks" sheetId="5" r:id="rId5"/>
     <sheet name="Sources &amp; Version" sheetId="6" r:id="rId6"/>
   </sheets>
+  <definedNames>
+    <definedName name="RateYears">tblRates[year_of_income]</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -284,7 +287,7 @@
     <t>2019-05</t>
   </si>
   <si>
-    <t>RBA statistical table F5 Indicator Lending Rates, series FILRHLBVS (Housing loans; Banks; Variable; Standard; Owner-occupier), figure for May 2019; cross-checked against the published Division 7A benchmark rate table.</t>
+    <t>RBA statistical table F5 Indicator Lending Rates, series FILRHLBVS (Housing loans; Banks; Variable; Standard; Owner-occupier), figure for May 2019; cross-checked against the published Division 7A benchmark rate table. Automated comparison 23 September 2026: xl/worksheets/sheet1.xml!D736, series identifier D11.</t>
   </si>
   <si>
     <t>2026-08-28</t>
@@ -293,31 +296,31 @@
     <t>2020-05</t>
   </si>
   <si>
-    <t>RBA statistical table F5 Indicator Lending Rates, series FILRHLBVS (Housing loans; Banks; Variable; Standard; Owner-occupier), figure for May 2020; cross-checked against the published Division 7A benchmark rate table.</t>
+    <t>RBA statistical table F5 Indicator Lending Rates, series FILRHLBVS (Housing loans; Banks; Variable; Standard; Owner-occupier), figure for May 2020; cross-checked against the published Division 7A benchmark rate table. Automated comparison 23 September 2026: xl/worksheets/sheet1.xml!D748, series identifier D11.</t>
   </si>
   <si>
     <t>2021-05</t>
   </si>
   <si>
-    <t>RBA statistical table F5 Indicator Lending Rates, series FILRHLBVS (Housing loans; Banks; Variable; Standard; Owner-occupier), figure for May 2021; cross-checked against the published Division 7A benchmark rate table.</t>
+    <t>RBA statistical table F5 Indicator Lending Rates, series FILRHLBVS (Housing loans; Banks; Variable; Standard; Owner-occupier), figure for May 2021; cross-checked against the published Division 7A benchmark rate table. Automated comparison 23 September 2026: xl/worksheets/sheet1.xml!D760, series identifier D11.</t>
   </si>
   <si>
     <t>2022-05</t>
   </si>
   <si>
-    <t>RBA statistical table F5 Indicator Lending Rates, series FILRHLBVS (Housing loans; Banks; Variable; Standard; Owner-occupier), figure for May 2022; cross-checked against the published Division 7A benchmark rate table.</t>
+    <t>RBA statistical table F5 Indicator Lending Rates, series FILRHLBVS (Housing loans; Banks; Variable; Standard; Owner-occupier), figure for May 2022; cross-checked against the published Division 7A benchmark rate table. Automated comparison 23 September 2026: xl/worksheets/sheet1.xml!D772, series identifier D11.</t>
   </si>
   <si>
     <t>2023-05</t>
   </si>
   <si>
-    <t>RBA statistical table F5 Indicator Lending Rates, series FILRHLBVS (Housing loans; Banks; Variable; Standard; Owner-occupier), figure for May 2023; cross-checked against the published Division 7A benchmark rate table.</t>
+    <t>RBA statistical table F5 Indicator Lending Rates, series FILRHLBVS (Housing loans; Banks; Variable; Standard; Owner-occupier), figure for May 2023; cross-checked against the published Division 7A benchmark rate table. Automated comparison 23 September 2026: xl/worksheets/sheet1.xml!D784, series identifier D11.</t>
   </si>
   <si>
     <t>2024-05</t>
   </si>
   <si>
-    <t>RBA statistical table F5 Indicator Lending Rates, series FILRHLBVS (Housing loans; Banks; Variable; Standard; Owner-occupier), figure for May 2024; cross-checked against the published Division 7A benchmark rate table.</t>
+    <t>RBA statistical table F5 Indicator Lending Rates, series FILRHLBVS (Housing loans; Banks; Variable; Standard; Owner-occupier), figure for May 2024; cross-checked against the published Division 7A benchmark rate table. Automated comparison 23 September 2026: xl/worksheets/sheet1.xml!D796, series identifier D11.</t>
   </si>
   <si>
     <t>2025-26</t>
@@ -326,7 +329,7 @@
     <t>2025-05</t>
   </si>
   <si>
-    <t>RBA statistical table F5 Indicator Lending Rates, series FILRHLBVS (Housing loans; Banks; Variable; Standard; Owner-occupier), figure for May 2025 (8.37 per cent). June 2025 was 8.27 per cent and is not the benchmark rate: it was published after the year of income began.</t>
+    <t>RBA statistical table F5 Indicator Lending Rates, series FILRHLBVS (Housing loans; Banks; Variable; Standard; Owner-occupier), figure for May 2025 (8.37 per cent). June 2025 was 8.27 per cent and is not the benchmark rate: it was published after the year of income began. Automated comparison 23 September 2026: xl/worksheets/sheet1.xml!D808, series identifier D11.</t>
   </si>
   <si>
     <t>2026-27</t>
@@ -335,7 +338,7 @@
     <t>2026-05</t>
   </si>
   <si>
-    <t>RBA statistical table F5 Indicator Lending Rates, series FILRHLBVS (Housing loans; Banks; Variable; Standard; Owner-occupier), figure for May 2026; cross-checked against the published Division 7A benchmark rate table.</t>
+    <t>RBA statistical table F5 Indicator Lending Rates, series FILRHLBVS (Housing loans; Banks; Variable; Standard; Owner-occupier), figure for May 2026; cross-checked against the published Division 7A benchmark rate table. Automated comparison 23 September 2026: xl/worksheets/sheet1.xml!D820, series identifier D11.</t>
   </si>
   <si>
     <t>To review a year outside this table, add a row with the May RBA F5 FILRHLBVS figure and cite where you read it. A blank source is not a review.</t>
@@ -2677,19 +2680,12 @@
       <formula>"PASS"</formula>
     </cfRule>
   </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" sqref="B2" xr:uid="{00000000-0002-0000-0300-000000000000}">
+      <formula1>RateYears</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
-        <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0300-000000000000}">
-          <x14:formula1>
-            <xm:f>Rates!$A$2:$A$9</xm:f>
-          </x14:formula1>
-          <xm:sqref>B2</xm:sqref>
-        </x14:dataValidation>
-      </x14:dataValidations>
-    </ext>
-  </extLst>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Cite the fixed compilation in the div7a workbook's Law source row
The builder still wrote the latest link into Sources & Version, so the shipped workbook and every later rebuild disagreed with the rest of the package. The builder now writes the 1 July 2026 compilation URL. The workbook was rebuilt with desktop Excel, and a cell-by-cell comparison with the previous file, covering formulas and cached values, differs only in that cell.
</commit_message>
<xml_diff>
--- a/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
+++ b/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
@@ -6,9 +6,9 @@
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B9C2A8D-EFF4-4CA2-B3A4-A1B9462A8FCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCADA3D8-7F1E-47BB-A0D5-4DDDC5C79244}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="390" windowWidth="38700" windowHeight="15885" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Start Here" sheetId="1" r:id="rId1"/>
@@ -464,7 +464,7 @@
     <t>Law source</t>
   </si>
   <si>
-    <t>https://www.legislation.gov.au/C1936A00027/latest/text</t>
+    <t>https://www.legislation.gov.au/C1936A00027/2026-07-01/text</t>
   </si>
   <si>
     <t>Benchmark rates</t>

</xml_diff>

<commit_message>
Cite the fixed 1 July 2026 ITAA 1936 compilation in div7a-loan-review (#295)
The primary source review, evaluation pack, README and workbook Law source row now link the 1 July 2026 compilation of C1936A00027 instead of the moving latest version. The workbook was rebuilt with desktop Excel and differs from the previous file only in that cell.
</commit_message>
<xml_diff>
--- a/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
+++ b/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
@@ -6,9 +6,9 @@
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B9C2A8D-EFF4-4CA2-B3A4-A1B9462A8FCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCADA3D8-7F1E-47BB-A0D5-4DDDC5C79244}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="390" windowWidth="38700" windowHeight="15885" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Start Here" sheetId="1" r:id="rId1"/>
@@ -464,7 +464,7 @@
     <t>Law source</t>
   </si>
   <si>
-    <t>https://www.legislation.gov.au/C1936A00027/latest/text</t>
+    <t>https://www.legislation.gov.au/C1936A00027/2026-07-01/text</t>
   </si>
   <si>
     <t>Benchmark rates</t>

</xml_diff>

<commit_message>
Release payday-super-checker 0.1.9, solomons-sword 0.1.10, the-wip-tally 0.1.3 and div7a-loan-review 0.1.6
Version bumps, release notes, rebuilt payday and Division 7A workbooks, and locks for the fixes merged from 27 to 30 September (#307, #318, #325, #326, #328, #329, #330).
</commit_message>
<xml_diff>
--- a/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
+++ b/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
@@ -6,7 +6,7 @@
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7A343B9-BA30-4589-8A19-80F1D424C2AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA5602AC-2D1F-441A-A40D-B6882D24FF72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="-105" windowWidth="26010" windowHeight="21705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -65,7 +65,7 @@
     <t>Overall status</t>
   </si>
   <si>
-    <t>div7a-loan-review workbook, engine 0.1.5. Macro-free. Not advice; see DISCLAIMER.md in the repository.</t>
+    <t>div7a-loan-review workbook, engine 0.1.6. Macro-free. Not advice; see DISCLAIMER.md in the repository.</t>
   </si>
   <si>
     <t>loan_id</t>
@@ -449,7 +449,7 @@
     <t>Workbook engine version</t>
   </si>
   <si>
-    <t>0.1.5</t>
+    <t>0.1.6</t>
   </si>
   <si>
     <t>Desktop Excel build used to calculate cached values</t>

</xml_diff>

<commit_message>
Release div7a-loan-review 0.2.0 and solomons-sword 0.2.0
Both ship #344's malformed-input fixes and the Python 3.11 floor from
#351. A floor raise changes the installation contract, so both move to
0.2.0; 0.1.6 and 0.1.10 remain the last releases for Python 3.10.

Each moves its version in pyproject.toml, the test literals and the
README, gains a RELEASE_NOTES.md section and its lock version line;
div7a-loan-review also moves __init__.py and CITATION.cff, and its
workbook was rebuilt with tools/build_workbook.py in desktop Excel so
Sources!B2 carries 0.2.0. The MCP's Division 7A test and quick-proof
literal follow the workspace engine, as in #332. The MCP still pins
div7a-loan-review 0.1.6 until 0.2.0 is on PyPI.
</commit_message>
<xml_diff>
--- a/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
+++ b/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA5602AC-2D1F-441A-A40D-B6882D24FF72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EEF1D6C-F520-48A2-B9FD-4356743E2E3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="26010" windowHeight="21705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-210" windowWidth="26010" windowHeight="21705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Start Here" sheetId="1" r:id="rId1"/>
@@ -65,7 +65,7 @@
     <t>Overall status</t>
   </si>
   <si>
-    <t>div7a-loan-review workbook, engine 0.1.6. Macro-free. Not advice; see DISCLAIMER.md in the repository.</t>
+    <t>div7a-loan-review workbook, engine 0.2.0. Macro-free. Not advice; see DISCLAIMER.md in the repository.</t>
   </si>
   <si>
     <t>loan_id</t>
@@ -449,7 +449,7 @@
     <t>Workbook engine version</t>
   </si>
   <si>
-    <t>0.1.6</t>
+    <t>0.2.0</t>
   </si>
   <si>
     <t>Desktop Excel build used to calculate cached values</t>
@@ -491,7 +491,7 @@
     <t>Experimental review aid. Not a Division 7A determination, not an ATO assessment, and not tax, legal or financial advice.</t>
   </si>
   <si>
-    <t>Excel 16.0 build 20430</t>
+    <t>Excel 16.0 build 20527</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Release div7a-loan-review 0.2.0 and solomons-sword 0.2.0 (#353)
Both ship #344's malformed-input fixes and the Python 3.11 floor from
#351. A floor raise changes the installation contract, so both move to
0.2.0; 0.1.6 and 0.1.10 remain the last releases for Python 3.10.

Each moves its version in pyproject.toml, the test literals and the
README, gains a RELEASE_NOTES.md section and its lock version line;
div7a-loan-review also moves __init__.py and CITATION.cff, and its
workbook was rebuilt with tools/build_workbook.py in desktop Excel so
Sources!B2 carries 0.2.0. The MCP's Division 7A test and quick-proof
literal follow the workspace engine, as in #332. The MCP still pins
div7a-loan-review 0.1.6 until 0.2.0 is on PyPI.
</commit_message>
<xml_diff>
--- a/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
+++ b/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA5602AC-2D1F-441A-A40D-B6882D24FF72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EEF1D6C-F520-48A2-B9FD-4356743E2E3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="26010" windowHeight="21705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-210" windowWidth="26010" windowHeight="21705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Start Here" sheetId="1" r:id="rId1"/>
@@ -65,7 +65,7 @@
     <t>Overall status</t>
   </si>
   <si>
-    <t>div7a-loan-review workbook, engine 0.1.6. Macro-free. Not advice; see DISCLAIMER.md in the repository.</t>
+    <t>div7a-loan-review workbook, engine 0.2.0. Macro-free. Not advice; see DISCLAIMER.md in the repository.</t>
   </si>
   <si>
     <t>loan_id</t>
@@ -449,7 +449,7 @@
     <t>Workbook engine version</t>
   </si>
   <si>
-    <t>0.1.6</t>
+    <t>0.2.0</t>
   </si>
   <si>
     <t>Desktop Excel build used to calculate cached values</t>
@@ -491,7 +491,7 @@
     <t>Experimental review aid. Not a Division 7A determination, not an ATO assessment, and not tax, legal or financial advice.</t>
   </si>
   <si>
-    <t>Excel 16.0 build 20430</t>
+    <t>Excel 16.0 build 20527</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Read Div7A workbook year labels the way the engine does
The workbook trimmed only ordinary spaces around a year of income, so a label
with a surrounding tab or non-breaking space failed in Excel while the engine
accepted it, and an internal tab could be erased into a valid label. Both
year columns now go through hidden helper columns that replace Python's
str.strip whitespace with spaces before trimming, so internal whitespace
still fails. When neither register year is known the gate is UNKNOWN and the
maximum term is blank. The workbook is rebuilt with desktop Excel.
</commit_message>
<xml_diff>
--- a/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
+++ b/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
@@ -6,7 +6,7 @@
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EEF1D6C-F520-48A2-B9FD-4356743E2E3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94D73362-5F24-42C3-95CE-6300FBA1E771}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="-210" windowWidth="26010" windowHeight="21705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="153">
   <si>
     <t>Division 7A loan review: s 109N terms and s 109E minimum yearly repayment</t>
   </si>
@@ -174,6 +174,12 @@
   </si>
   <si>
     <t>Sample_row</t>
+  </si>
+  <si>
+    <t>Year_made_text</t>
+  </si>
+  <si>
+    <t>Year_tested_text</t>
   </si>
   <si>
     <t>L-101</t>
@@ -676,8 +682,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblLoans" displayName="tblLoans" ref="A1:AJ9">
-  <tableColumns count="36">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblLoans" displayName="tblLoans" ref="A1:AL9">
+  <tableColumns count="38">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="loan_id"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="borrower_reference"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="year_loan_made"/>
@@ -693,10 +699,10 @@
     <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="out_of_scope_reason"/>
     <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="year_of_income_being_tested"/>
     <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Status">
-      <calculatedColumnFormula>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","SKIPPED",IF(IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;1998,FALSE),"SKIPPED","REVIEWED"))</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","SKIPPED",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&lt;1998,FALSE),"SKIPPED","REVIEWED"))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Floor_year">
-      <calculatedColumnFormula>IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_tested_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),tblLoans[[#This Row],[Year_made_text]],tblLoans[[#This Row],[Year_tested_text]])</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Floor_rate">
       <calculatedColumnFormula>IFERROR(INDEX(tblRates[rate],MATCH(tblLoans[[#This Row],[Floor_year]],tblRates[year_of_income],0)),"")</calculatedColumnFormula>
@@ -720,10 +726,10 @@
       <calculatedColumnFormula>IF(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),"UNKNOWN",IF(tblLoans[[#This Row],[Allowed_term_raw]]="",IF(tblLoans[[#This Row],[maximum_term_years]]&lt;=7,"PASS","UNKNOWN"),IF(tblLoans[[#This Row],[maximum_term_years]]&lt;=tblLoans[[#This Row],[Allowed_term_raw]],"PASS","FAIL")))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="24" xr3:uid="{00000000-0010-0000-0000-000018000000}" name="Gate_verdict">
-      <calculatedColumnFormula>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Limb_a_written]]="FAIL",tblLoans[[#This Row],[Limb_lodgment]]="FAIL",tblLoans[[#This Row],[Limb_b_rate]]="FAIL",tblLoans[[#This Row],[Limb_c_term]]="FAIL"),"NOT_COMPLYING",IF(OR(tblLoans[[#This Row],[Limb_a_written]]="UNKNOWN",tblLoans[[#This Row],[Limb_lodgment]]="UNKNOWN",tblLoans[[#This Row],[Limb_b_rate]]="UNKNOWN",tblLoans[[#This Row],[Limb_c_term]]="UNKNOWN"),"UNKNOWN","COMPLYING")))</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[Floor_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"UNKNOWN",IF(OR(tblLoans[[#This Row],[Limb_a_written]]="FAIL",tblLoans[[#This Row],[Limb_lodgment]]="FAIL",tblLoans[[#This Row],[Limb_b_rate]]="FAIL",tblLoans[[#This Row],[Limb_c_term]]="FAIL"),"NOT_COMPLYING",IF(OR(tblLoans[[#This Row],[Limb_a_written]]="UNKNOWN",tblLoans[[#This Row],[Limb_lodgment]]="UNKNOWN",tblLoans[[#This Row],[Limb_b_rate]]="UNKNOWN",tblLoans[[#This Row],[Limb_c_term]]="UNKNOWN"),"UNKNOWN","COMPLYING"))))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="25" xr3:uid="{00000000-0010-0000-0000-000019000000}" name="Max_term_allowed">
-      <calculatedColumnFormula>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(tblLoans[[#This Row],[Allowed_term_raw]]&lt;&gt;"",tblLoans[[#This Row],[Allowed_term_raw]],IF(AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),tblLoans[[#This Row],[maximum_term_years]]&lt;=7),7,"")))</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(OR(tblLoans[[#This Row],[Status]]="SKIPPED",OR(LOWER(TRIM(tblLoans[[#This Row],[Floor_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),"",IF(tblLoans[[#This Row],[Allowed_term_raw]]&lt;&gt;"",tblLoans[[#This Row],[Allowed_term_raw]],IF(AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),tblLoans[[#This Row],[maximum_term_years]]&lt;=7),7,"")))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="26" xr3:uid="{00000000-0010-0000-0000-00001A000000}" name="Term_used">
       <calculatedColumnFormula>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),ROUNDUP(tblLoans[[#This Row],[remaining_term_years]],0),""))</calculatedColumnFormula>
@@ -732,10 +738,10 @@
       <calculatedColumnFormula>IF(AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),ISNUMBER(Summary!$B$3),Summary!$B$3&gt;0,ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&gt;0),ROUND(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]*Summary!$B$3/(1-(1/(1+Summary!$B$3))^tblLoans[[#This Row],[Term_used]]),2),"")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="28" xr3:uid="{00000000-0010-0000-0000-00001C000000}" name="MYR_verdict">
-      <calculatedColumnFormula>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")),TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")=Summary!$B$2,IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_made_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[Year_made_text]]),tblLoans[[#This Row],[Year_made_text]]=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_made_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="29" xr3:uid="{00000000-0010-0000-0000-00001D000000}" name="MYR_reason">
-      <calculatedColumnFormula>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),"gate benchmark year differs from year_loan_made",IF(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[Year_made_text]],"gate benchmark year differs from year_loan_made",IF(tblLoans[[#This Row],[Year_made_text]]=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_made_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="30" xr3:uid="{00000000-0010-0000-0000-00001E000000}" name="MYR_required">
       <calculatedColumnFormula>IF(OR(tblLoans[[#This Row],[MYR_verdict]]="MYR_MET",tblLoans[[#This Row],[MYR_verdict]]="MYR_SHORT"),tblLoans[[#This Row],[MYR_raw]],"")</calculatedColumnFormula>
@@ -753,10 +759,16 @@
       <calculatedColumnFormula>IF(OR(_xlfn.ISFORMULA(tblLoans[[#This Row],[loan_id]]),_xlfn.ISFORMULA(tblLoans[[#This Row],[borrower_reference]]),_xlfn.ISFORMULA(tblLoans[[#This Row],[year_loan_made]]),_xlfn.ISFORMULA(tblLoans[[#This Row],[written_agreement]]),_xlfn.ISFORMULA(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]),_xlfn.ISFORMULA(tblLoans[[#This Row],[maximum_term_years]]),_xlfn.ISFORMULA(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]),_xlfn.ISFORMULA(tblLoans[[#This Row],[security_coverage_at_first_made]]),_xlfn.ISFORMULA(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),_xlfn.ISFORMULA(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),_xlfn.ISFORMULA(tblLoans[[#This Row],[remaining_term_years]]),_xlfn.ISFORMULA(tblLoans[[#This Row],[payments_applied_during_the_year]]),_xlfn.ISFORMULA(tblLoans[[#This Row],[out_of_scope_reason]]),_xlfn.ISFORMULA(tblLoans[[#This Row],[year_of_income_being_tested]])),1,0)</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="35" xr3:uid="{00000000-0010-0000-0000-000023000000}" name="Input_problem">
-      <calculatedColumnFormula>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[payments_applied_during_the_year]]),N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_made_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[Year_made_text]])=7,MID(tblLoans[[#This Row],[Year_made_text]],5,1)="-",ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],1,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],2,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],3,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],4,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],6,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],7,1))),VALUE(RIGHT(tblLoans[[#This Row],[Year_made_text]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))+1,100),VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&gt;=1900,VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_tested_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[Year_tested_text]])=7,MID(tblLoans[[#This Row],[Year_tested_text]],5,1)="-",ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],1,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],2,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],3,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],4,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],6,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],7,1))),VALUE(RIGHT(tblLoans[[#This Row],[Year_tested_text]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[Year_tested_text]],4))+1,100),VALUE(LEFT(tblLoans[[#This Row],[Year_tested_text]],4))&gt;=1900,VALUE(LEFT(tblLoans[[#This Row],[Year_tested_text]],4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[payments_applied_during_the_year]]),N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="36" xr3:uid="{00000000-0010-0000-0000-000024000000}" name="Sample_row">
-      <calculatedColumnFormula>IF(SUMPRODUCT((tblLoans[[#This Row],[loan_id]]&amp;""={"L-101","L-102","L-103","L-104","L-105","L-106","L-107","L-108"})*(tblLoans[[#This Row],[year_loan_made]]&amp;""={"2023-24","2022-23","2021-22","2024-25","2019-20","2020-21","2023-24","1996-97"}))&gt;0,1,0)</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(SUMPRODUCT((tblLoans[[#This Row],[loan_id]]&amp;""={"L-101","L-102","L-103","L-104","L-105","L-106","L-107","L-108"})*(tblLoans[[#This Row],[Year_made_text]]&amp;""={"2023-24","2022-23","2021-22","2024-25","2019-20","2020-21","2023-24","1996-97"}))&gt;0,1,0)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="37" xr3:uid="{00000000-0010-0000-0000-000025000000}" name="Year_made_text">
+      <calculatedColumnFormula>TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(tblLoans[[#This Row],[year_loan_made]]&amp;"",_xlfn.UNICHAR(9)," "),_xlfn.UNICHAR(10)," "),_xlfn.UNICHAR(11)," "),_xlfn.UNICHAR(12)," "),_xlfn.UNICHAR(13)," "),_xlfn.UNICHAR(28)," "),_xlfn.UNICHAR(29)," "),_xlfn.UNICHAR(30)," "),_xlfn.UNICHAR(31)," "),_xlfn.UNICHAR(133)," "),_xlfn.UNICHAR(160)," "),_xlfn.UNICHAR(5760)," "),_xlfn.UNICHAR(8192)," "),_xlfn.UNICHAR(8193)," "),_xlfn.UNICHAR(8194)," "),_xlfn.UNICHAR(8195)," "),_xlfn.UNICHAR(8196)," "),_xlfn.UNICHAR(8197)," "),_xlfn.UNICHAR(8198)," "),_xlfn.UNICHAR(8199)," "),_xlfn.UNICHAR(8200)," "),_xlfn.UNICHAR(8201)," "),_xlfn.UNICHAR(8202)," "),_xlfn.UNICHAR(8232)," "),_xlfn.UNICHAR(8233)," "),_xlfn.UNICHAR(8239)," "),_xlfn.UNICHAR(8287)," "),_xlfn.UNICHAR(12288)," "))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="38" xr3:uid="{00000000-0010-0000-0000-000026000000}" name="Year_tested_text">
+      <calculatedColumnFormula>TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;"",_xlfn.UNICHAR(9)," "),_xlfn.UNICHAR(10)," "),_xlfn.UNICHAR(11)," "),_xlfn.UNICHAR(12)," "),_xlfn.UNICHAR(13)," "),_xlfn.UNICHAR(28)," "),_xlfn.UNICHAR(29)," "),_xlfn.UNICHAR(30)," "),_xlfn.UNICHAR(31)," "),_xlfn.UNICHAR(133)," "),_xlfn.UNICHAR(160)," "),_xlfn.UNICHAR(5760)," "),_xlfn.UNICHAR(8192)," "),_xlfn.UNICHAR(8193)," "),_xlfn.UNICHAR(8194)," "),_xlfn.UNICHAR(8195)," "),_xlfn.UNICHAR(8196)," "),_xlfn.UNICHAR(8197)," "),_xlfn.UNICHAR(8198)," "),_xlfn.UNICHAR(8199)," "),_xlfn.UNICHAR(8200)," "),_xlfn.UNICHAR(8201)," "),_xlfn.UNICHAR(8202)," "),_xlfn.UNICHAR(8232)," "),_xlfn.UNICHAR(8233)," "),_xlfn.UNICHAR(8239)," "),_xlfn.UNICHAR(8287)," "),_xlfn.UNICHAR(12288)," "))</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1138,7 +1150,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:AJ9"/>
+  <dimension ref="A1:AL9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -1151,9 +1163,10 @@
     <col min="29" max="29" width="40" customWidth="1"/>
     <col min="30" max="32" width="14" customWidth="1"/>
     <col min="33" max="36" width="12" customWidth="1"/>
+    <col min="37" max="38" width="12" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>9</v>
       </c>
@@ -1262,31 +1275,37 @@
       <c r="AJ1" s="5" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK1" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="AL1" s="5" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F2" s="7">
         <v>7</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H2" s="7" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I2" s="7">
         <v>8.2699999999999996E-2</v>
@@ -1303,11 +1322,11 @@
       <c r="M2" s="6"/>
       <c r="N2" s="6"/>
       <c r="O2" s="9" t="str">
-        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","SKIPPED",IF(IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;1998,FALSE),"SKIPPED","REVIEWED"))</f>
+        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","SKIPPED",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&lt;1998,FALSE),"SKIPPED","REVIEWED"))</f>
         <v>REVIEWED</v>
       </c>
       <c r="P2" s="9" t="str">
-        <f>IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))</f>
+        <f>IF(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_tested_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),tblLoans[[#This Row],[Year_made_text]],tblLoans[[#This Row],[Year_tested_text]])</f>
         <v>2023-24</v>
       </c>
       <c r="Q2" s="9">
@@ -1339,11 +1358,11 @@
         <v>PASS</v>
       </c>
       <c r="X2" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Limb_a_written]]="FAIL",tblLoans[[#This Row],[Limb_lodgment]]="FAIL",tblLoans[[#This Row],[Limb_b_rate]]="FAIL",tblLoans[[#This Row],[Limb_c_term]]="FAIL"),"NOT_COMPLYING",IF(OR(tblLoans[[#This Row],[Limb_a_written]]="UNKNOWN",tblLoans[[#This Row],[Limb_lodgment]]="UNKNOWN",tblLoans[[#This Row],[Limb_b_rate]]="UNKNOWN",tblLoans[[#This Row],[Limb_c_term]]="UNKNOWN"),"UNKNOWN","COMPLYING")))</f>
+        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[Floor_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"UNKNOWN",IF(OR(tblLoans[[#This Row],[Limb_a_written]]="FAIL",tblLoans[[#This Row],[Limb_lodgment]]="FAIL",tblLoans[[#This Row],[Limb_b_rate]]="FAIL",tblLoans[[#This Row],[Limb_c_term]]="FAIL"),"NOT_COMPLYING",IF(OR(tblLoans[[#This Row],[Limb_a_written]]="UNKNOWN",tblLoans[[#This Row],[Limb_lodgment]]="UNKNOWN",tblLoans[[#This Row],[Limb_b_rate]]="UNKNOWN",tblLoans[[#This Row],[Limb_c_term]]="UNKNOWN"),"UNKNOWN","COMPLYING"))))</f>
         <v>COMPLYING</v>
       </c>
       <c r="Y2" s="9">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(tblLoans[[#This Row],[Allowed_term_raw]]&lt;&gt;"",tblLoans[[#This Row],[Allowed_term_raw]],IF(AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),tblLoans[[#This Row],[maximum_term_years]]&lt;=7),7,"")))</f>
+        <f>IF(OR(tblLoans[[#This Row],[Status]]="SKIPPED",OR(LOWER(TRIM(tblLoans[[#This Row],[Floor_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),"",IF(tblLoans[[#This Row],[Allowed_term_raw]]&lt;&gt;"",tblLoans[[#This Row],[Allowed_term_raw]],IF(AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),tblLoans[[#This Row],[maximum_term_years]]&lt;=7),7,"")))</f>
         <v>7</v>
       </c>
       <c r="Z2" s="9">
@@ -1355,11 +1374,11 @@
         <v>47212.37</v>
       </c>
       <c r="AB2" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")),TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")=Summary!$B$2,IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
+        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_made_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[Year_made_text]]),tblLoans[[#This Row],[Year_made_text]]=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_made_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
         <v>MYR_SHORT</v>
       </c>
       <c r="AC2" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),"gate benchmark year differs from year_loan_made",IF(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
+        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[Year_made_text]],"gate benchmark year differs from year_loan_made",IF(tblLoans[[#This Row],[Year_made_text]]=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_made_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
         <v/>
       </c>
       <c r="AD2" s="10">
@@ -1383,38 +1402,46 @@
         <v>0</v>
       </c>
       <c r="AI2" s="9" t="str">
-        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[payments_applied_during_the_year]]),N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</f>
+        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_made_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[Year_made_text]])=7,MID(tblLoans[[#This Row],[Year_made_text]],5,1)="-",ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],1,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],2,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],3,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],4,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],6,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],7,1))),VALUE(RIGHT(tblLoans[[#This Row],[Year_made_text]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))+1,100),VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&gt;=1900,VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_tested_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[Year_tested_text]])=7,MID(tblLoans[[#This Row],[Year_tested_text]],5,1)="-",ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],1,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],2,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],3,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],4,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],6,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],7,1))),VALUE(RIGHT(tblLoans[[#This Row],[Year_tested_text]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[Year_tested_text]],4))+1,100),VALUE(LEFT(tblLoans[[#This Row],[Year_tested_text]],4))&gt;=1900,VALUE(LEFT(tblLoans[[#This Row],[Year_tested_text]],4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[payments_applied_during_the_year]]),N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</f>
         <v/>
       </c>
       <c r="AJ2" s="9">
-        <f>IF(SUMPRODUCT((tblLoans[[#This Row],[loan_id]]&amp;""={"L-101","L-102","L-103","L-104","L-105","L-106","L-107","L-108"})*(tblLoans[[#This Row],[year_loan_made]]&amp;""={"2023-24","2022-23","2021-22","2024-25","2019-20","2020-21","2023-24","1996-97"}))&gt;0,1,0)</f>
+        <f>IF(SUMPRODUCT((tblLoans[[#This Row],[loan_id]]&amp;""={"L-101","L-102","L-103","L-104","L-105","L-106","L-107","L-108"})*(tblLoans[[#This Row],[Year_made_text]]&amp;""={"2023-24","2022-23","2021-22","2024-25","2019-20","2020-21","2023-24","1996-97"}))&gt;0,1,0)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK2" s="9" t="str">
+        <f>TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(tblLoans[[#This Row],[year_loan_made]]&amp;"",_xlfn.UNICHAR(9)," "),_xlfn.UNICHAR(10)," "),_xlfn.UNICHAR(11)," "),_xlfn.UNICHAR(12)," "),_xlfn.UNICHAR(13)," "),_xlfn.UNICHAR(28)," "),_xlfn.UNICHAR(29)," "),_xlfn.UNICHAR(30)," "),_xlfn.UNICHAR(31)," "),_xlfn.UNICHAR(133)," "),_xlfn.UNICHAR(160)," "),_xlfn.UNICHAR(5760)," "),_xlfn.UNICHAR(8192)," "),_xlfn.UNICHAR(8193)," "),_xlfn.UNICHAR(8194)," "),_xlfn.UNICHAR(8195)," "),_xlfn.UNICHAR(8196)," "),_xlfn.UNICHAR(8197)," "),_xlfn.UNICHAR(8198)," "),_xlfn.UNICHAR(8199)," "),_xlfn.UNICHAR(8200)," "),_xlfn.UNICHAR(8201)," "),_xlfn.UNICHAR(8202)," "),_xlfn.UNICHAR(8232)," "),_xlfn.UNICHAR(8233)," "),_xlfn.UNICHAR(8239)," "),_xlfn.UNICHAR(8287)," "),_xlfn.UNICHAR(12288)," "))</f>
+        <v>2023-24</v>
+      </c>
+      <c r="AL2" s="9" t="str">
+        <f>TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;"",_xlfn.UNICHAR(9)," "),_xlfn.UNICHAR(10)," "),_xlfn.UNICHAR(11)," "),_xlfn.UNICHAR(12)," "),_xlfn.UNICHAR(13)," "),_xlfn.UNICHAR(28)," "),_xlfn.UNICHAR(29)," "),_xlfn.UNICHAR(30)," "),_xlfn.UNICHAR(31)," "),_xlfn.UNICHAR(133)," "),_xlfn.UNICHAR(160)," "),_xlfn.UNICHAR(5760)," "),_xlfn.UNICHAR(8192)," "),_xlfn.UNICHAR(8193)," "),_xlfn.UNICHAR(8194)," "),_xlfn.UNICHAR(8195)," "),_xlfn.UNICHAR(8196)," "),_xlfn.UNICHAR(8197)," "),_xlfn.UNICHAR(8198)," "),_xlfn.UNICHAR(8199)," "),_xlfn.UNICHAR(8200)," "),_xlfn.UNICHAR(8201)," "),_xlfn.UNICHAR(8202)," "),_xlfn.UNICHAR(8232)," "),_xlfn.UNICHAR(8233)," "),_xlfn.UNICHAR(8239)," "),_xlfn.UNICHAR(8287)," "),_xlfn.UNICHAR(12288)," "))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F3" s="7">
         <v>7</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I3" s="7">
         <v>0.04</v>
@@ -1431,11 +1458,11 @@
       <c r="M3" s="6"/>
       <c r="N3" s="6"/>
       <c r="O3" s="9" t="str">
-        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","SKIPPED",IF(IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;1998,FALSE),"SKIPPED","REVIEWED"))</f>
+        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","SKIPPED",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&lt;1998,FALSE),"SKIPPED","REVIEWED"))</f>
         <v>REVIEWED</v>
       </c>
       <c r="P3" s="9" t="str">
-        <f>IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))</f>
+        <f>IF(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_tested_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),tblLoans[[#This Row],[Year_made_text]],tblLoans[[#This Row],[Year_tested_text]])</f>
         <v>2022-23</v>
       </c>
       <c r="Q3" s="9">
@@ -1467,11 +1494,11 @@
         <v>PASS</v>
       </c>
       <c r="X3" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Limb_a_written]]="FAIL",tblLoans[[#This Row],[Limb_lodgment]]="FAIL",tblLoans[[#This Row],[Limb_b_rate]]="FAIL",tblLoans[[#This Row],[Limb_c_term]]="FAIL"),"NOT_COMPLYING",IF(OR(tblLoans[[#This Row],[Limb_a_written]]="UNKNOWN",tblLoans[[#This Row],[Limb_lodgment]]="UNKNOWN",tblLoans[[#This Row],[Limb_b_rate]]="UNKNOWN",tblLoans[[#This Row],[Limb_c_term]]="UNKNOWN"),"UNKNOWN","COMPLYING")))</f>
+        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[Floor_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"UNKNOWN",IF(OR(tblLoans[[#This Row],[Limb_a_written]]="FAIL",tblLoans[[#This Row],[Limb_lodgment]]="FAIL",tblLoans[[#This Row],[Limb_b_rate]]="FAIL",tblLoans[[#This Row],[Limb_c_term]]="FAIL"),"NOT_COMPLYING",IF(OR(tblLoans[[#This Row],[Limb_a_written]]="UNKNOWN",tblLoans[[#This Row],[Limb_lodgment]]="UNKNOWN",tblLoans[[#This Row],[Limb_b_rate]]="UNKNOWN",tblLoans[[#This Row],[Limb_c_term]]="UNKNOWN"),"UNKNOWN","COMPLYING"))))</f>
         <v>NOT_COMPLYING</v>
       </c>
       <c r="Y3" s="9">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(tblLoans[[#This Row],[Allowed_term_raw]]&lt;&gt;"",tblLoans[[#This Row],[Allowed_term_raw]],IF(AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),tblLoans[[#This Row],[maximum_term_years]]&lt;=7),7,"")))</f>
+        <f>IF(OR(tblLoans[[#This Row],[Status]]="SKIPPED",OR(LOWER(TRIM(tblLoans[[#This Row],[Floor_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),"",IF(tblLoans[[#This Row],[Allowed_term_raw]]&lt;&gt;"",tblLoans[[#This Row],[Allowed_term_raw]],IF(AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),tblLoans[[#This Row],[maximum_term_years]]&lt;=7),7,"")))</f>
         <v>7</v>
       </c>
       <c r="Z3" s="9">
@@ -1483,11 +1510,11 @@
         <v>27640.06</v>
       </c>
       <c r="AB3" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")),TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")=Summary!$B$2,IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
+        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_made_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[Year_made_text]]),tblLoans[[#This Row],[Year_made_text]]=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_made_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
         <v>REFUSED</v>
       </c>
       <c r="AC3" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),"gate benchmark year differs from year_loan_made",IF(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
+        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[Year_made_text]],"gate benchmark year differs from year_loan_made",IF(tblLoans[[#This Row],[Year_made_text]]=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_made_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
         <v>s 109N gate is NOT_COMPLYING, so s 109E produces no repayment figure</v>
       </c>
       <c r="AD3" s="10" t="str">
@@ -1511,38 +1538,46 @@
         <v>0</v>
       </c>
       <c r="AI3" s="9" t="str">
-        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[payments_applied_during_the_year]]),N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</f>
+        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_made_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[Year_made_text]])=7,MID(tblLoans[[#This Row],[Year_made_text]],5,1)="-",ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],1,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],2,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],3,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],4,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],6,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],7,1))),VALUE(RIGHT(tblLoans[[#This Row],[Year_made_text]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))+1,100),VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&gt;=1900,VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_tested_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[Year_tested_text]])=7,MID(tblLoans[[#This Row],[Year_tested_text]],5,1)="-",ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],1,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],2,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],3,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],4,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],6,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],7,1))),VALUE(RIGHT(tblLoans[[#This Row],[Year_tested_text]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[Year_tested_text]],4))+1,100),VALUE(LEFT(tblLoans[[#This Row],[Year_tested_text]],4))&gt;=1900,VALUE(LEFT(tblLoans[[#This Row],[Year_tested_text]],4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[payments_applied_during_the_year]]),N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</f>
         <v/>
       </c>
       <c r="AJ3" s="9">
-        <f>IF(SUMPRODUCT((tblLoans[[#This Row],[loan_id]]&amp;""={"L-101","L-102","L-103","L-104","L-105","L-106","L-107","L-108"})*(tblLoans[[#This Row],[year_loan_made]]&amp;""={"2023-24","2022-23","2021-22","2024-25","2019-20","2020-21","2023-24","1996-97"}))&gt;0,1,0)</f>
+        <f>IF(SUMPRODUCT((tblLoans[[#This Row],[loan_id]]&amp;""={"L-101","L-102","L-103","L-104","L-105","L-106","L-107","L-108"})*(tblLoans[[#This Row],[Year_made_text]]&amp;""={"2023-24","2022-23","2021-22","2024-25","2019-20","2020-21","2023-24","1996-97"}))&gt;0,1,0)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK3" s="9" t="str">
+        <f>TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(tblLoans[[#This Row],[year_loan_made]]&amp;"",_xlfn.UNICHAR(9)," "),_xlfn.UNICHAR(10)," "),_xlfn.UNICHAR(11)," "),_xlfn.UNICHAR(12)," "),_xlfn.UNICHAR(13)," "),_xlfn.UNICHAR(28)," "),_xlfn.UNICHAR(29)," "),_xlfn.UNICHAR(30)," "),_xlfn.UNICHAR(31)," "),_xlfn.UNICHAR(133)," "),_xlfn.UNICHAR(160)," "),_xlfn.UNICHAR(5760)," "),_xlfn.UNICHAR(8192)," "),_xlfn.UNICHAR(8193)," "),_xlfn.UNICHAR(8194)," "),_xlfn.UNICHAR(8195)," "),_xlfn.UNICHAR(8196)," "),_xlfn.UNICHAR(8197)," "),_xlfn.UNICHAR(8198)," "),_xlfn.UNICHAR(8199)," "),_xlfn.UNICHAR(8200)," "),_xlfn.UNICHAR(8201)," "),_xlfn.UNICHAR(8202)," "),_xlfn.UNICHAR(8232)," "),_xlfn.UNICHAR(8233)," "),_xlfn.UNICHAR(8239)," "),_xlfn.UNICHAR(8287)," "),_xlfn.UNICHAR(12288)," "))</f>
+        <v>2022-23</v>
+      </c>
+      <c r="AL3" s="9" t="str">
+        <f>TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;"",_xlfn.UNICHAR(9)," "),_xlfn.UNICHAR(10)," "),_xlfn.UNICHAR(11)," "),_xlfn.UNICHAR(12)," "),_xlfn.UNICHAR(13)," "),_xlfn.UNICHAR(28)," "),_xlfn.UNICHAR(29)," "),_xlfn.UNICHAR(30)," "),_xlfn.UNICHAR(31)," "),_xlfn.UNICHAR(133)," "),_xlfn.UNICHAR(160)," "),_xlfn.UNICHAR(5760)," "),_xlfn.UNICHAR(8192)," "),_xlfn.UNICHAR(8193)," "),_xlfn.UNICHAR(8194)," "),_xlfn.UNICHAR(8195)," "),_xlfn.UNICHAR(8196)," "),_xlfn.UNICHAR(8197)," "),_xlfn.UNICHAR(8198)," "),_xlfn.UNICHAR(8199)," "),_xlfn.UNICHAR(8200)," "),_xlfn.UNICHAR(8201)," "),_xlfn.UNICHAR(8202)," "),_xlfn.UNICHAR(8232)," "),_xlfn.UNICHAR(8233)," "),_xlfn.UNICHAR(8239)," "),_xlfn.UNICHAR(8287)," "),_xlfn.UNICHAR(12288)," "))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D4" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="E4" s="7" t="s">
         <v>50</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>48</v>
       </c>
       <c r="F4" s="7">
         <v>7</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I4" s="7">
         <v>4.5199999999999997E-2</v>
@@ -1559,11 +1594,11 @@
       <c r="M4" s="6"/>
       <c r="N4" s="6"/>
       <c r="O4" s="9" t="str">
-        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","SKIPPED",IF(IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;1998,FALSE),"SKIPPED","REVIEWED"))</f>
+        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","SKIPPED",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&lt;1998,FALSE),"SKIPPED","REVIEWED"))</f>
         <v>REVIEWED</v>
       </c>
       <c r="P4" s="9" t="str">
-        <f>IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))</f>
+        <f>IF(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_tested_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),tblLoans[[#This Row],[Year_made_text]],tblLoans[[#This Row],[Year_tested_text]])</f>
         <v>2021-22</v>
       </c>
       <c r="Q4" s="9">
@@ -1595,11 +1630,11 @@
         <v>PASS</v>
       </c>
       <c r="X4" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Limb_a_written]]="FAIL",tblLoans[[#This Row],[Limb_lodgment]]="FAIL",tblLoans[[#This Row],[Limb_b_rate]]="FAIL",tblLoans[[#This Row],[Limb_c_term]]="FAIL"),"NOT_COMPLYING",IF(OR(tblLoans[[#This Row],[Limb_a_written]]="UNKNOWN",tblLoans[[#This Row],[Limb_lodgment]]="UNKNOWN",tblLoans[[#This Row],[Limb_b_rate]]="UNKNOWN",tblLoans[[#This Row],[Limb_c_term]]="UNKNOWN"),"UNKNOWN","COMPLYING")))</f>
+        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[Floor_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"UNKNOWN",IF(OR(tblLoans[[#This Row],[Limb_a_written]]="FAIL",tblLoans[[#This Row],[Limb_lodgment]]="FAIL",tblLoans[[#This Row],[Limb_b_rate]]="FAIL",tblLoans[[#This Row],[Limb_c_term]]="FAIL"),"NOT_COMPLYING",IF(OR(tblLoans[[#This Row],[Limb_a_written]]="UNKNOWN",tblLoans[[#This Row],[Limb_lodgment]]="UNKNOWN",tblLoans[[#This Row],[Limb_b_rate]]="UNKNOWN",tblLoans[[#This Row],[Limb_c_term]]="UNKNOWN"),"UNKNOWN","COMPLYING"))))</f>
         <v>UNKNOWN</v>
       </c>
       <c r="Y4" s="9">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(tblLoans[[#This Row],[Allowed_term_raw]]&lt;&gt;"",tblLoans[[#This Row],[Allowed_term_raw]],IF(AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),tblLoans[[#This Row],[maximum_term_years]]&lt;=7),7,"")))</f>
+        <f>IF(OR(tblLoans[[#This Row],[Status]]="SKIPPED",OR(LOWER(TRIM(tblLoans[[#This Row],[Floor_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),"",IF(tblLoans[[#This Row],[Allowed_term_raw]]&lt;&gt;"",tblLoans[[#This Row],[Allowed_term_raw]],IF(AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),tblLoans[[#This Row],[maximum_term_years]]&lt;=7),7,"")))</f>
         <v>7</v>
       </c>
       <c r="Z4" s="9">
@@ -1611,11 +1646,11 @@
         <v>28334.799999999999</v>
       </c>
       <c r="AB4" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")),TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")=Summary!$B$2,IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
+        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_made_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[Year_made_text]]),tblLoans[[#This Row],[Year_made_text]]=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_made_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
         <v>REFUSED</v>
       </c>
       <c r="AC4" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),"gate benchmark year differs from year_loan_made",IF(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
+        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[Year_made_text]],"gate benchmark year differs from year_loan_made",IF(tblLoans[[#This Row],[Year_made_text]]=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_made_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
         <v>s 109N gate is UNKNOWN, so s 109E produces no repayment figure</v>
       </c>
       <c r="AD4" s="10" t="str">
@@ -1639,38 +1674,46 @@
         <v>0</v>
       </c>
       <c r="AI4" s="9" t="str">
-        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[payments_applied_during_the_year]]),N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</f>
+        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_made_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[Year_made_text]])=7,MID(tblLoans[[#This Row],[Year_made_text]],5,1)="-",ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],1,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],2,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],3,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],4,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],6,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],7,1))),VALUE(RIGHT(tblLoans[[#This Row],[Year_made_text]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))+1,100),VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&gt;=1900,VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_tested_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[Year_tested_text]])=7,MID(tblLoans[[#This Row],[Year_tested_text]],5,1)="-",ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],1,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],2,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],3,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],4,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],6,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],7,1))),VALUE(RIGHT(tblLoans[[#This Row],[Year_tested_text]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[Year_tested_text]],4))+1,100),VALUE(LEFT(tblLoans[[#This Row],[Year_tested_text]],4))&gt;=1900,VALUE(LEFT(tblLoans[[#This Row],[Year_tested_text]],4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[payments_applied_during_the_year]]),N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</f>
         <v/>
       </c>
       <c r="AJ4" s="9">
-        <f>IF(SUMPRODUCT((tblLoans[[#This Row],[loan_id]]&amp;""={"L-101","L-102","L-103","L-104","L-105","L-106","L-107","L-108"})*(tblLoans[[#This Row],[year_loan_made]]&amp;""={"2023-24","2022-23","2021-22","2024-25","2019-20","2020-21","2023-24","1996-97"}))&gt;0,1,0)</f>
+        <f>IF(SUMPRODUCT((tblLoans[[#This Row],[loan_id]]&amp;""={"L-101","L-102","L-103","L-104","L-105","L-106","L-107","L-108"})*(tblLoans[[#This Row],[Year_made_text]]&amp;""={"2023-24","2022-23","2021-22","2024-25","2019-20","2020-21","2023-24","1996-97"}))&gt;0,1,0)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK4" s="9" t="str">
+        <f>TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(tblLoans[[#This Row],[year_loan_made]]&amp;"",_xlfn.UNICHAR(9)," "),_xlfn.UNICHAR(10)," "),_xlfn.UNICHAR(11)," "),_xlfn.UNICHAR(12)," "),_xlfn.UNICHAR(13)," "),_xlfn.UNICHAR(28)," "),_xlfn.UNICHAR(29)," "),_xlfn.UNICHAR(30)," "),_xlfn.UNICHAR(31)," "),_xlfn.UNICHAR(133)," "),_xlfn.UNICHAR(160)," "),_xlfn.UNICHAR(5760)," "),_xlfn.UNICHAR(8192)," "),_xlfn.UNICHAR(8193)," "),_xlfn.UNICHAR(8194)," "),_xlfn.UNICHAR(8195)," "),_xlfn.UNICHAR(8196)," "),_xlfn.UNICHAR(8197)," "),_xlfn.UNICHAR(8198)," "),_xlfn.UNICHAR(8199)," "),_xlfn.UNICHAR(8200)," "),_xlfn.UNICHAR(8201)," "),_xlfn.UNICHAR(8202)," "),_xlfn.UNICHAR(8232)," "),_xlfn.UNICHAR(8233)," "),_xlfn.UNICHAR(8239)," "),_xlfn.UNICHAR(8287)," "),_xlfn.UNICHAR(12288)," "))</f>
+        <v>2021-22</v>
+      </c>
+      <c r="AL4" s="9" t="str">
+        <f>TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;"",_xlfn.UNICHAR(9)," "),_xlfn.UNICHAR(10)," "),_xlfn.UNICHAR(11)," "),_xlfn.UNICHAR(12)," "),_xlfn.UNICHAR(13)," "),_xlfn.UNICHAR(28)," "),_xlfn.UNICHAR(29)," "),_xlfn.UNICHAR(30)," "),_xlfn.UNICHAR(31)," "),_xlfn.UNICHAR(133)," "),_xlfn.UNICHAR(160)," "),_xlfn.UNICHAR(5760)," "),_xlfn.UNICHAR(8192)," "),_xlfn.UNICHAR(8193)," "),_xlfn.UNICHAR(8194)," "),_xlfn.UNICHAR(8195)," "),_xlfn.UNICHAR(8196)," "),_xlfn.UNICHAR(8197)," "),_xlfn.UNICHAR(8198)," "),_xlfn.UNICHAR(8199)," "),_xlfn.UNICHAR(8200)," "),_xlfn.UNICHAR(8201)," "),_xlfn.UNICHAR(8202)," "),_xlfn.UNICHAR(8232)," "),_xlfn.UNICHAR(8233)," "),_xlfn.UNICHAR(8239)," "),_xlfn.UNICHAR(8287)," "),_xlfn.UNICHAR(12288)," "))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F5" s="7">
         <v>7</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I5" s="7">
         <v>8.77E-2</v>
@@ -1682,16 +1725,16 @@
         <v>5</v>
       </c>
       <c r="L5" s="8" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="M5" s="6"/>
       <c r="N5" s="6"/>
       <c r="O5" s="9" t="str">
-        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","SKIPPED",IF(IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;1998,FALSE),"SKIPPED","REVIEWED"))</f>
+        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","SKIPPED",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&lt;1998,FALSE),"SKIPPED","REVIEWED"))</f>
         <v>REVIEWED</v>
       </c>
       <c r="P5" s="9" t="str">
-        <f>IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))</f>
+        <f>IF(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_tested_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),tblLoans[[#This Row],[Year_made_text]],tblLoans[[#This Row],[Year_tested_text]])</f>
         <v>2024-25</v>
       </c>
       <c r="Q5" s="9">
@@ -1723,11 +1766,11 @@
         <v>PASS</v>
       </c>
       <c r="X5" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Limb_a_written]]="FAIL",tblLoans[[#This Row],[Limb_lodgment]]="FAIL",tblLoans[[#This Row],[Limb_b_rate]]="FAIL",tblLoans[[#This Row],[Limb_c_term]]="FAIL"),"NOT_COMPLYING",IF(OR(tblLoans[[#This Row],[Limb_a_written]]="UNKNOWN",tblLoans[[#This Row],[Limb_lodgment]]="UNKNOWN",tblLoans[[#This Row],[Limb_b_rate]]="UNKNOWN",tblLoans[[#This Row],[Limb_c_term]]="UNKNOWN"),"UNKNOWN","COMPLYING")))</f>
+        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[Floor_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"UNKNOWN",IF(OR(tblLoans[[#This Row],[Limb_a_written]]="FAIL",tblLoans[[#This Row],[Limb_lodgment]]="FAIL",tblLoans[[#This Row],[Limb_b_rate]]="FAIL",tblLoans[[#This Row],[Limb_c_term]]="FAIL"),"NOT_COMPLYING",IF(OR(tblLoans[[#This Row],[Limb_a_written]]="UNKNOWN",tblLoans[[#This Row],[Limb_lodgment]]="UNKNOWN",tblLoans[[#This Row],[Limb_b_rate]]="UNKNOWN",tblLoans[[#This Row],[Limb_c_term]]="UNKNOWN"),"UNKNOWN","COMPLYING"))))</f>
         <v>COMPLYING</v>
       </c>
       <c r="Y5" s="9">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(tblLoans[[#This Row],[Allowed_term_raw]]&lt;&gt;"",tblLoans[[#This Row],[Allowed_term_raw]],IF(AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),tblLoans[[#This Row],[maximum_term_years]]&lt;=7),7,"")))</f>
+        <f>IF(OR(tblLoans[[#This Row],[Status]]="SKIPPED",OR(LOWER(TRIM(tblLoans[[#This Row],[Floor_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),"",IF(tblLoans[[#This Row],[Allowed_term_raw]]&lt;&gt;"",tblLoans[[#This Row],[Allowed_term_raw]],IF(AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),tblLoans[[#This Row],[maximum_term_years]]&lt;=7),7,"")))</f>
         <v>7</v>
       </c>
       <c r="Z5" s="9">
@@ -1739,11 +1782,11 @@
         <v>22489.279999999999</v>
       </c>
       <c r="AB5" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")),TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")=Summary!$B$2,IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
+        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_made_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[Year_made_text]]),tblLoans[[#This Row],[Year_made_text]]=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_made_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
         <v>UNKNOWN</v>
       </c>
       <c r="AC5" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),"gate benchmark year differs from year_loan_made",IF(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
+        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[Year_made_text]],"gate benchmark year differs from year_loan_made",IF(tblLoans[[#This Row],[Year_made_text]]=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_made_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
         <v>payments applied not established</v>
       </c>
       <c r="AD5" s="10" t="str">
@@ -1767,38 +1810,46 @@
         <v>0</v>
       </c>
       <c r="AI5" s="9" t="str">
-        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[payments_applied_during_the_year]]),N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</f>
+        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_made_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[Year_made_text]])=7,MID(tblLoans[[#This Row],[Year_made_text]],5,1)="-",ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],1,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],2,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],3,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],4,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],6,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],7,1))),VALUE(RIGHT(tblLoans[[#This Row],[Year_made_text]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))+1,100),VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&gt;=1900,VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_tested_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[Year_tested_text]])=7,MID(tblLoans[[#This Row],[Year_tested_text]],5,1)="-",ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],1,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],2,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],3,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],4,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],6,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],7,1))),VALUE(RIGHT(tblLoans[[#This Row],[Year_tested_text]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[Year_tested_text]],4))+1,100),VALUE(LEFT(tblLoans[[#This Row],[Year_tested_text]],4))&gt;=1900,VALUE(LEFT(tblLoans[[#This Row],[Year_tested_text]],4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[payments_applied_during_the_year]]),N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</f>
         <v/>
       </c>
       <c r="AJ5" s="9">
-        <f>IF(SUMPRODUCT((tblLoans[[#This Row],[loan_id]]&amp;""={"L-101","L-102","L-103","L-104","L-105","L-106","L-107","L-108"})*(tblLoans[[#This Row],[year_loan_made]]&amp;""={"2023-24","2022-23","2021-22","2024-25","2019-20","2020-21","2023-24","1996-97"}))&gt;0,1,0)</f>
+        <f>IF(SUMPRODUCT((tblLoans[[#This Row],[loan_id]]&amp;""={"L-101","L-102","L-103","L-104","L-105","L-106","L-107","L-108"})*(tblLoans[[#This Row],[Year_made_text]]&amp;""={"2023-24","2022-23","2021-22","2024-25","2019-20","2020-21","2023-24","1996-97"}))&gt;0,1,0)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK5" s="9" t="str">
+        <f>TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(tblLoans[[#This Row],[year_loan_made]]&amp;"",_xlfn.UNICHAR(9)," "),_xlfn.UNICHAR(10)," "),_xlfn.UNICHAR(11)," "),_xlfn.UNICHAR(12)," "),_xlfn.UNICHAR(13)," "),_xlfn.UNICHAR(28)," "),_xlfn.UNICHAR(29)," "),_xlfn.UNICHAR(30)," "),_xlfn.UNICHAR(31)," "),_xlfn.UNICHAR(133)," "),_xlfn.UNICHAR(160)," "),_xlfn.UNICHAR(5760)," "),_xlfn.UNICHAR(8192)," "),_xlfn.UNICHAR(8193)," "),_xlfn.UNICHAR(8194)," "),_xlfn.UNICHAR(8195)," "),_xlfn.UNICHAR(8196)," "),_xlfn.UNICHAR(8197)," "),_xlfn.UNICHAR(8198)," "),_xlfn.UNICHAR(8199)," "),_xlfn.UNICHAR(8200)," "),_xlfn.UNICHAR(8201)," "),_xlfn.UNICHAR(8202)," "),_xlfn.UNICHAR(8232)," "),_xlfn.UNICHAR(8233)," "),_xlfn.UNICHAR(8239)," "),_xlfn.UNICHAR(8287)," "),_xlfn.UNICHAR(12288)," "))</f>
+        <v>2024-25</v>
+      </c>
+      <c r="AL5" s="9" t="str">
+        <f>TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;"",_xlfn.UNICHAR(9)," "),_xlfn.UNICHAR(10)," "),_xlfn.UNICHAR(11)," "),_xlfn.UNICHAR(12)," "),_xlfn.UNICHAR(13)," "),_xlfn.UNICHAR(28)," "),_xlfn.UNICHAR(29)," "),_xlfn.UNICHAR(30)," "),_xlfn.UNICHAR(31)," "),_xlfn.UNICHAR(133)," "),_xlfn.UNICHAR(160)," "),_xlfn.UNICHAR(5760)," "),_xlfn.UNICHAR(8192)," "),_xlfn.UNICHAR(8193)," "),_xlfn.UNICHAR(8194)," "),_xlfn.UNICHAR(8195)," "),_xlfn.UNICHAR(8196)," "),_xlfn.UNICHAR(8197)," "),_xlfn.UNICHAR(8198)," "),_xlfn.UNICHAR(8199)," "),_xlfn.UNICHAR(8200)," "),_xlfn.UNICHAR(8201)," "),_xlfn.UNICHAR(8202)," "),_xlfn.UNICHAR(8232)," "),_xlfn.UNICHAR(8233)," "),_xlfn.UNICHAR(8239)," "),_xlfn.UNICHAR(8287)," "),_xlfn.UNICHAR(12288)," "))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F6" s="7">
         <v>7</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I6" s="7">
         <v>5.3699999999999998E-2</v>
@@ -1815,11 +1866,11 @@
       <c r="M6" s="6"/>
       <c r="N6" s="6"/>
       <c r="O6" s="9" t="str">
-        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","SKIPPED",IF(IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;1998,FALSE),"SKIPPED","REVIEWED"))</f>
+        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","SKIPPED",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&lt;1998,FALSE),"SKIPPED","REVIEWED"))</f>
         <v>REVIEWED</v>
       </c>
       <c r="P6" s="9" t="str">
-        <f>IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))</f>
+        <f>IF(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_tested_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),tblLoans[[#This Row],[Year_made_text]],tblLoans[[#This Row],[Year_tested_text]])</f>
         <v>2019-20</v>
       </c>
       <c r="Q6" s="9">
@@ -1851,11 +1902,11 @@
         <v>PASS</v>
       </c>
       <c r="X6" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Limb_a_written]]="FAIL",tblLoans[[#This Row],[Limb_lodgment]]="FAIL",tblLoans[[#This Row],[Limb_b_rate]]="FAIL",tblLoans[[#This Row],[Limb_c_term]]="FAIL"),"NOT_COMPLYING",IF(OR(tblLoans[[#This Row],[Limb_a_written]]="UNKNOWN",tblLoans[[#This Row],[Limb_lodgment]]="UNKNOWN",tblLoans[[#This Row],[Limb_b_rate]]="UNKNOWN",tblLoans[[#This Row],[Limb_c_term]]="UNKNOWN"),"UNKNOWN","COMPLYING")))</f>
+        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[Floor_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"UNKNOWN",IF(OR(tblLoans[[#This Row],[Limb_a_written]]="FAIL",tblLoans[[#This Row],[Limb_lodgment]]="FAIL",tblLoans[[#This Row],[Limb_b_rate]]="FAIL",tblLoans[[#This Row],[Limb_c_term]]="FAIL"),"NOT_COMPLYING",IF(OR(tblLoans[[#This Row],[Limb_a_written]]="UNKNOWN",tblLoans[[#This Row],[Limb_lodgment]]="UNKNOWN",tblLoans[[#This Row],[Limb_b_rate]]="UNKNOWN",tblLoans[[#This Row],[Limb_c_term]]="UNKNOWN"),"UNKNOWN","COMPLYING"))))</f>
         <v>COMPLYING</v>
       </c>
       <c r="Y6" s="9">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(tblLoans[[#This Row],[Allowed_term_raw]]&lt;&gt;"",tblLoans[[#This Row],[Allowed_term_raw]],IF(AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),tblLoans[[#This Row],[maximum_term_years]]&lt;=7),7,"")))</f>
+        <f>IF(OR(tblLoans[[#This Row],[Status]]="SKIPPED",OR(LOWER(TRIM(tblLoans[[#This Row],[Floor_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),"",IF(tblLoans[[#This Row],[Allowed_term_raw]]&lt;&gt;"",tblLoans[[#This Row],[Allowed_term_raw]],IF(AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),tblLoans[[#This Row],[maximum_term_years]]&lt;=7),7,"")))</f>
         <v>7</v>
       </c>
       <c r="Z6" s="9">
@@ -1867,11 +1918,11 @@
         <v/>
       </c>
       <c r="AB6" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")),TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")=Summary!$B$2,IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
+        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_made_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[Year_made_text]]),tblLoans[[#This Row],[Year_made_text]]=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_made_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
         <v>REFUSED</v>
       </c>
       <c r="AC6" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),"gate benchmark year differs from year_loan_made",IF(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
+        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[Year_made_text]],"gate benchmark year differs from year_loan_made",IF(tblLoans[[#This Row],[Year_made_text]]=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_made_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
         <v>nil remaining term under s 109E(6)</v>
       </c>
       <c r="AD6" s="10" t="str">
@@ -1895,35 +1946,43 @@
         <v>0</v>
       </c>
       <c r="AI6" s="9" t="str">
-        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[payments_applied_during_the_year]]),N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</f>
+        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_made_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[Year_made_text]])=7,MID(tblLoans[[#This Row],[Year_made_text]],5,1)="-",ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],1,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],2,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],3,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],4,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],6,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],7,1))),VALUE(RIGHT(tblLoans[[#This Row],[Year_made_text]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))+1,100),VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&gt;=1900,VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_tested_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[Year_tested_text]])=7,MID(tblLoans[[#This Row],[Year_tested_text]],5,1)="-",ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],1,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],2,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],3,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],4,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],6,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],7,1))),VALUE(RIGHT(tblLoans[[#This Row],[Year_tested_text]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[Year_tested_text]],4))+1,100),VALUE(LEFT(tblLoans[[#This Row],[Year_tested_text]],4))&gt;=1900,VALUE(LEFT(tblLoans[[#This Row],[Year_tested_text]],4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[payments_applied_during_the_year]]),N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</f>
         <v/>
       </c>
       <c r="AJ6" s="9">
-        <f>IF(SUMPRODUCT((tblLoans[[#This Row],[loan_id]]&amp;""={"L-101","L-102","L-103","L-104","L-105","L-106","L-107","L-108"})*(tblLoans[[#This Row],[year_loan_made]]&amp;""={"2023-24","2022-23","2021-22","2024-25","2019-20","2020-21","2023-24","1996-97"}))&gt;0,1,0)</f>
+        <f>IF(SUMPRODUCT((tblLoans[[#This Row],[loan_id]]&amp;""={"L-101","L-102","L-103","L-104","L-105","L-106","L-107","L-108"})*(tblLoans[[#This Row],[Year_made_text]]&amp;""={"2023-24","2022-23","2021-22","2024-25","2019-20","2020-21","2023-24","1996-97"}))&gt;0,1,0)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK6" s="9" t="str">
+        <f>TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(tblLoans[[#This Row],[year_loan_made]]&amp;"",_xlfn.UNICHAR(9)," "),_xlfn.UNICHAR(10)," "),_xlfn.UNICHAR(11)," "),_xlfn.UNICHAR(12)," "),_xlfn.UNICHAR(13)," "),_xlfn.UNICHAR(28)," "),_xlfn.UNICHAR(29)," "),_xlfn.UNICHAR(30)," "),_xlfn.UNICHAR(31)," "),_xlfn.UNICHAR(133)," "),_xlfn.UNICHAR(160)," "),_xlfn.UNICHAR(5760)," "),_xlfn.UNICHAR(8192)," "),_xlfn.UNICHAR(8193)," "),_xlfn.UNICHAR(8194)," "),_xlfn.UNICHAR(8195)," "),_xlfn.UNICHAR(8196)," "),_xlfn.UNICHAR(8197)," "),_xlfn.UNICHAR(8198)," "),_xlfn.UNICHAR(8199)," "),_xlfn.UNICHAR(8200)," "),_xlfn.UNICHAR(8201)," "),_xlfn.UNICHAR(8202)," "),_xlfn.UNICHAR(8232)," "),_xlfn.UNICHAR(8233)," "),_xlfn.UNICHAR(8239)," "),_xlfn.UNICHAR(8287)," "),_xlfn.UNICHAR(12288)," "))</f>
+        <v>2019-20</v>
+      </c>
+      <c r="AL6" s="9" t="str">
+        <f>TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;"",_xlfn.UNICHAR(9)," "),_xlfn.UNICHAR(10)," "),_xlfn.UNICHAR(11)," "),_xlfn.UNICHAR(12)," "),_xlfn.UNICHAR(13)," "),_xlfn.UNICHAR(28)," "),_xlfn.UNICHAR(29)," "),_xlfn.UNICHAR(30)," "),_xlfn.UNICHAR(31)," "),_xlfn.UNICHAR(133)," "),_xlfn.UNICHAR(160)," "),_xlfn.UNICHAR(5760)," "),_xlfn.UNICHAR(8192)," "),_xlfn.UNICHAR(8193)," "),_xlfn.UNICHAR(8194)," "),_xlfn.UNICHAR(8195)," "),_xlfn.UNICHAR(8196)," "),_xlfn.UNICHAR(8197)," "),_xlfn.UNICHAR(8198)," "),_xlfn.UNICHAR(8199)," "),_xlfn.UNICHAR(8200)," "),_xlfn.UNICHAR(8201)," "),_xlfn.UNICHAR(8202)," "),_xlfn.UNICHAR(8232)," "),_xlfn.UNICHAR(8233)," "),_xlfn.UNICHAR(8239)," "),_xlfn.UNICHAR(8287)," "),_xlfn.UNICHAR(12288)," "))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F7" s="7">
         <v>25</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H7" s="7">
         <v>1.0900000000000001</v>
@@ -1943,11 +2002,11 @@
       <c r="M7" s="6"/>
       <c r="N7" s="6"/>
       <c r="O7" s="9" t="str">
-        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","SKIPPED",IF(IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;1998,FALSE),"SKIPPED","REVIEWED"))</f>
+        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","SKIPPED",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&lt;1998,FALSE),"SKIPPED","REVIEWED"))</f>
         <v>REVIEWED</v>
       </c>
       <c r="P7" s="9" t="str">
-        <f>IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))</f>
+        <f>IF(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_tested_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),tblLoans[[#This Row],[Year_made_text]],tblLoans[[#This Row],[Year_tested_text]])</f>
         <v>2020-21</v>
       </c>
       <c r="Q7" s="9">
@@ -1979,11 +2038,11 @@
         <v>FAIL</v>
       </c>
       <c r="X7" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Limb_a_written]]="FAIL",tblLoans[[#This Row],[Limb_lodgment]]="FAIL",tblLoans[[#This Row],[Limb_b_rate]]="FAIL",tblLoans[[#This Row],[Limb_c_term]]="FAIL"),"NOT_COMPLYING",IF(OR(tblLoans[[#This Row],[Limb_a_written]]="UNKNOWN",tblLoans[[#This Row],[Limb_lodgment]]="UNKNOWN",tblLoans[[#This Row],[Limb_b_rate]]="UNKNOWN",tblLoans[[#This Row],[Limb_c_term]]="UNKNOWN"),"UNKNOWN","COMPLYING")))</f>
+        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[Floor_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"UNKNOWN",IF(OR(tblLoans[[#This Row],[Limb_a_written]]="FAIL",tblLoans[[#This Row],[Limb_lodgment]]="FAIL",tblLoans[[#This Row],[Limb_b_rate]]="FAIL",tblLoans[[#This Row],[Limb_c_term]]="FAIL"),"NOT_COMPLYING",IF(OR(tblLoans[[#This Row],[Limb_a_written]]="UNKNOWN",tblLoans[[#This Row],[Limb_lodgment]]="UNKNOWN",tblLoans[[#This Row],[Limb_b_rate]]="UNKNOWN",tblLoans[[#This Row],[Limb_c_term]]="UNKNOWN"),"UNKNOWN","COMPLYING"))))</f>
         <v>NOT_COMPLYING</v>
       </c>
       <c r="Y7" s="9">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(tblLoans[[#This Row],[Allowed_term_raw]]&lt;&gt;"",tblLoans[[#This Row],[Allowed_term_raw]],IF(AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),tblLoans[[#This Row],[maximum_term_years]]&lt;=7),7,"")))</f>
+        <f>IF(OR(tblLoans[[#This Row],[Status]]="SKIPPED",OR(LOWER(TRIM(tblLoans[[#This Row],[Floor_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),"",IF(tblLoans[[#This Row],[Allowed_term_raw]]&lt;&gt;"",tblLoans[[#This Row],[Allowed_term_raw]],IF(AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),tblLoans[[#This Row],[maximum_term_years]]&lt;=7),7,"")))</f>
         <v>7</v>
       </c>
       <c r="Z7" s="9">
@@ -1995,11 +2054,11 @@
         <v>36713.81</v>
       </c>
       <c r="AB7" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")),TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")=Summary!$B$2,IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
+        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_made_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[Year_made_text]]),tblLoans[[#This Row],[Year_made_text]]=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_made_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
         <v>REFUSED</v>
       </c>
       <c r="AC7" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),"gate benchmark year differs from year_loan_made",IF(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
+        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[Year_made_text]],"gate benchmark year differs from year_loan_made",IF(tblLoans[[#This Row],[Year_made_text]]=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_made_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
         <v>s 109N gate is NOT_COMPLYING, so s 109E produces no repayment figure</v>
       </c>
       <c r="AD7" s="10" t="str">
@@ -2023,61 +2082,69 @@
         <v>0</v>
       </c>
       <c r="AI7" s="9" t="str">
-        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[payments_applied_during_the_year]]),N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</f>
+        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_made_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[Year_made_text]])=7,MID(tblLoans[[#This Row],[Year_made_text]],5,1)="-",ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],1,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],2,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],3,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],4,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],6,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],7,1))),VALUE(RIGHT(tblLoans[[#This Row],[Year_made_text]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))+1,100),VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&gt;=1900,VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_tested_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[Year_tested_text]])=7,MID(tblLoans[[#This Row],[Year_tested_text]],5,1)="-",ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],1,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],2,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],3,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],4,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],6,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],7,1))),VALUE(RIGHT(tblLoans[[#This Row],[Year_tested_text]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[Year_tested_text]],4))+1,100),VALUE(LEFT(tblLoans[[#This Row],[Year_tested_text]],4))&gt;=1900,VALUE(LEFT(tblLoans[[#This Row],[Year_tested_text]],4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[payments_applied_during_the_year]]),N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</f>
         <v/>
       </c>
       <c r="AJ7" s="9">
-        <f>IF(SUMPRODUCT((tblLoans[[#This Row],[loan_id]]&amp;""={"L-101","L-102","L-103","L-104","L-105","L-106","L-107","L-108"})*(tblLoans[[#This Row],[year_loan_made]]&amp;""={"2023-24","2022-23","2021-22","2024-25","2019-20","2020-21","2023-24","1996-97"}))&gt;0,1,0)</f>
+        <f>IF(SUMPRODUCT((tblLoans[[#This Row],[loan_id]]&amp;""={"L-101","L-102","L-103","L-104","L-105","L-106","L-107","L-108"})*(tblLoans[[#This Row],[Year_made_text]]&amp;""={"2023-24","2022-23","2021-22","2024-25","2019-20","2020-21","2023-24","1996-97"}))&gt;0,1,0)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK7" s="9" t="str">
+        <f>TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(tblLoans[[#This Row],[year_loan_made]]&amp;"",_xlfn.UNICHAR(9)," "),_xlfn.UNICHAR(10)," "),_xlfn.UNICHAR(11)," "),_xlfn.UNICHAR(12)," "),_xlfn.UNICHAR(13)," "),_xlfn.UNICHAR(28)," "),_xlfn.UNICHAR(29)," "),_xlfn.UNICHAR(30)," "),_xlfn.UNICHAR(31)," "),_xlfn.UNICHAR(133)," "),_xlfn.UNICHAR(160)," "),_xlfn.UNICHAR(5760)," "),_xlfn.UNICHAR(8192)," "),_xlfn.UNICHAR(8193)," "),_xlfn.UNICHAR(8194)," "),_xlfn.UNICHAR(8195)," "),_xlfn.UNICHAR(8196)," "),_xlfn.UNICHAR(8197)," "),_xlfn.UNICHAR(8198)," "),_xlfn.UNICHAR(8199)," "),_xlfn.UNICHAR(8200)," "),_xlfn.UNICHAR(8201)," "),_xlfn.UNICHAR(8202)," "),_xlfn.UNICHAR(8232)," "),_xlfn.UNICHAR(8233)," "),_xlfn.UNICHAR(8239)," "),_xlfn.UNICHAR(8287)," "),_xlfn.UNICHAR(12288)," "))</f>
+        <v>2020-21</v>
+      </c>
+      <c r="AL7" s="9" t="str">
+        <f>TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;"",_xlfn.UNICHAR(9)," "),_xlfn.UNICHAR(10)," "),_xlfn.UNICHAR(11)," "),_xlfn.UNICHAR(12)," "),_xlfn.UNICHAR(13)," "),_xlfn.UNICHAR(28)," "),_xlfn.UNICHAR(29)," "),_xlfn.UNICHAR(30)," "),_xlfn.UNICHAR(31)," "),_xlfn.UNICHAR(133)," "),_xlfn.UNICHAR(160)," "),_xlfn.UNICHAR(5760)," "),_xlfn.UNICHAR(8192)," "),_xlfn.UNICHAR(8193)," "),_xlfn.UNICHAR(8194)," "),_xlfn.UNICHAR(8195)," "),_xlfn.UNICHAR(8196)," "),_xlfn.UNICHAR(8197)," "),_xlfn.UNICHAR(8198)," "),_xlfn.UNICHAR(8199)," "),_xlfn.UNICHAR(8200)," "),_xlfn.UNICHAR(8201)," "),_xlfn.UNICHAR(8202)," "),_xlfn.UNICHAR(8232)," "),_xlfn.UNICHAR(8233)," "),_xlfn.UNICHAR(8239)," "),_xlfn.UNICHAR(8287)," "),_xlfn.UNICHAR(12288)," "))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I8" s="7" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="J8" s="8" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="K8" s="7" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="L8" s="8" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="M8" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="N8" s="6"/>
       <c r="O8" s="9" t="str">
-        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","SKIPPED",IF(IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;1998,FALSE),"SKIPPED","REVIEWED"))</f>
+        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","SKIPPED",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&lt;1998,FALSE),"SKIPPED","REVIEWED"))</f>
         <v>SKIPPED</v>
       </c>
       <c r="P8" s="9" t="str">
-        <f>IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))</f>
+        <f>IF(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_tested_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),tblLoans[[#This Row],[Year_made_text]],tblLoans[[#This Row],[Year_tested_text]])</f>
         <v>2023-24</v>
       </c>
       <c r="Q8" s="9">
@@ -2109,11 +2176,11 @@
         <v>UNKNOWN</v>
       </c>
       <c r="X8" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Limb_a_written]]="FAIL",tblLoans[[#This Row],[Limb_lodgment]]="FAIL",tblLoans[[#This Row],[Limb_b_rate]]="FAIL",tblLoans[[#This Row],[Limb_c_term]]="FAIL"),"NOT_COMPLYING",IF(OR(tblLoans[[#This Row],[Limb_a_written]]="UNKNOWN",tblLoans[[#This Row],[Limb_lodgment]]="UNKNOWN",tblLoans[[#This Row],[Limb_b_rate]]="UNKNOWN",tblLoans[[#This Row],[Limb_c_term]]="UNKNOWN"),"UNKNOWN","COMPLYING")))</f>
+        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[Floor_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"UNKNOWN",IF(OR(tblLoans[[#This Row],[Limb_a_written]]="FAIL",tblLoans[[#This Row],[Limb_lodgment]]="FAIL",tblLoans[[#This Row],[Limb_b_rate]]="FAIL",tblLoans[[#This Row],[Limb_c_term]]="FAIL"),"NOT_COMPLYING",IF(OR(tblLoans[[#This Row],[Limb_a_written]]="UNKNOWN",tblLoans[[#This Row],[Limb_lodgment]]="UNKNOWN",tblLoans[[#This Row],[Limb_b_rate]]="UNKNOWN",tblLoans[[#This Row],[Limb_c_term]]="UNKNOWN"),"UNKNOWN","COMPLYING"))))</f>
         <v/>
       </c>
       <c r="Y8" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(tblLoans[[#This Row],[Allowed_term_raw]]&lt;&gt;"",tblLoans[[#This Row],[Allowed_term_raw]],IF(AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),tblLoans[[#This Row],[maximum_term_years]]&lt;=7),7,"")))</f>
+        <f>IF(OR(tblLoans[[#This Row],[Status]]="SKIPPED",OR(LOWER(TRIM(tblLoans[[#This Row],[Floor_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),"",IF(tblLoans[[#This Row],[Allowed_term_raw]]&lt;&gt;"",tblLoans[[#This Row],[Allowed_term_raw]],IF(AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),tblLoans[[#This Row],[maximum_term_years]]&lt;=7),7,"")))</f>
         <v/>
       </c>
       <c r="Z8" s="9" t="str">
@@ -2125,11 +2192,11 @@
         <v/>
       </c>
       <c r="AB8" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")),TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")=Summary!$B$2,IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
+        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_made_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[Year_made_text]]),tblLoans[[#This Row],[Year_made_text]]=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_made_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
         <v/>
       </c>
       <c r="AC8" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),"gate benchmark year differs from year_loan_made",IF(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
+        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[Year_made_text]],"gate benchmark year differs from year_loan_made",IF(tblLoans[[#This Row],[Year_made_text]]=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_made_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
         <v/>
       </c>
       <c r="AD8" s="10" t="str">
@@ -2153,38 +2220,46 @@
         <v>0</v>
       </c>
       <c r="AI8" s="9" t="str">
-        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[payments_applied_during_the_year]]),N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</f>
+        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_made_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[Year_made_text]])=7,MID(tblLoans[[#This Row],[Year_made_text]],5,1)="-",ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],1,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],2,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],3,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],4,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],6,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],7,1))),VALUE(RIGHT(tblLoans[[#This Row],[Year_made_text]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))+1,100),VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&gt;=1900,VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_tested_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[Year_tested_text]])=7,MID(tblLoans[[#This Row],[Year_tested_text]],5,1)="-",ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],1,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],2,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],3,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],4,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],6,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],7,1))),VALUE(RIGHT(tblLoans[[#This Row],[Year_tested_text]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[Year_tested_text]],4))+1,100),VALUE(LEFT(tblLoans[[#This Row],[Year_tested_text]],4))&gt;=1900,VALUE(LEFT(tblLoans[[#This Row],[Year_tested_text]],4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[payments_applied_during_the_year]]),N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</f>
         <v/>
       </c>
       <c r="AJ8" s="9">
-        <f>IF(SUMPRODUCT((tblLoans[[#This Row],[loan_id]]&amp;""={"L-101","L-102","L-103","L-104","L-105","L-106","L-107","L-108"})*(tblLoans[[#This Row],[year_loan_made]]&amp;""={"2023-24","2022-23","2021-22","2024-25","2019-20","2020-21","2023-24","1996-97"}))&gt;0,1,0)</f>
+        <f>IF(SUMPRODUCT((tblLoans[[#This Row],[loan_id]]&amp;""={"L-101","L-102","L-103","L-104","L-105","L-106","L-107","L-108"})*(tblLoans[[#This Row],[Year_made_text]]&amp;""={"2023-24","2022-23","2021-22","2024-25","2019-20","2020-21","2023-24","1996-97"}))&gt;0,1,0)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AK8" s="9" t="str">
+        <f>TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(tblLoans[[#This Row],[year_loan_made]]&amp;"",_xlfn.UNICHAR(9)," "),_xlfn.UNICHAR(10)," "),_xlfn.UNICHAR(11)," "),_xlfn.UNICHAR(12)," "),_xlfn.UNICHAR(13)," "),_xlfn.UNICHAR(28)," "),_xlfn.UNICHAR(29)," "),_xlfn.UNICHAR(30)," "),_xlfn.UNICHAR(31)," "),_xlfn.UNICHAR(133)," "),_xlfn.UNICHAR(160)," "),_xlfn.UNICHAR(5760)," "),_xlfn.UNICHAR(8192)," "),_xlfn.UNICHAR(8193)," "),_xlfn.UNICHAR(8194)," "),_xlfn.UNICHAR(8195)," "),_xlfn.UNICHAR(8196)," "),_xlfn.UNICHAR(8197)," "),_xlfn.UNICHAR(8198)," "),_xlfn.UNICHAR(8199)," "),_xlfn.UNICHAR(8200)," "),_xlfn.UNICHAR(8201)," "),_xlfn.UNICHAR(8202)," "),_xlfn.UNICHAR(8232)," "),_xlfn.UNICHAR(8233)," "),_xlfn.UNICHAR(8239)," "),_xlfn.UNICHAR(8287)," "),_xlfn.UNICHAR(12288)," "))</f>
+        <v>2023-24</v>
+      </c>
+      <c r="AL8" s="9" t="str">
+        <f>TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;"",_xlfn.UNICHAR(9)," "),_xlfn.UNICHAR(10)," "),_xlfn.UNICHAR(11)," "),_xlfn.UNICHAR(12)," "),_xlfn.UNICHAR(13)," "),_xlfn.UNICHAR(28)," "),_xlfn.UNICHAR(29)," "),_xlfn.UNICHAR(30)," "),_xlfn.UNICHAR(31)," "),_xlfn.UNICHAR(133)," "),_xlfn.UNICHAR(160)," "),_xlfn.UNICHAR(5760)," "),_xlfn.UNICHAR(8192)," "),_xlfn.UNICHAR(8193)," "),_xlfn.UNICHAR(8194)," "),_xlfn.UNICHAR(8195)," "),_xlfn.UNICHAR(8196)," "),_xlfn.UNICHAR(8197)," "),_xlfn.UNICHAR(8198)," "),_xlfn.UNICHAR(8199)," "),_xlfn.UNICHAR(8200)," "),_xlfn.UNICHAR(8201)," "),_xlfn.UNICHAR(8202)," "),_xlfn.UNICHAR(8232)," "),_xlfn.UNICHAR(8233)," "),_xlfn.UNICHAR(8239)," "),_xlfn.UNICHAR(8287)," "),_xlfn.UNICHAR(12288)," "))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F9" s="7">
         <v>7</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I9" s="7">
         <v>7.0000000000000007E-2</v>
@@ -2201,11 +2276,11 @@
       <c r="M9" s="6"/>
       <c r="N9" s="6"/>
       <c r="O9" s="9" t="str">
-        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","SKIPPED",IF(IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;1998,FALSE),"SKIPPED","REVIEWED"))</f>
+        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","SKIPPED",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&lt;1998,FALSE),"SKIPPED","REVIEWED"))</f>
         <v>SKIPPED</v>
       </c>
       <c r="P9" s="9" t="str">
-        <f>IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))</f>
+        <f>IF(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_tested_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),tblLoans[[#This Row],[Year_made_text]],tblLoans[[#This Row],[Year_tested_text]])</f>
         <v>1996-97</v>
       </c>
       <c r="Q9" s="9" t="str">
@@ -2237,11 +2312,11 @@
         <v>PASS</v>
       </c>
       <c r="X9" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Limb_a_written]]="FAIL",tblLoans[[#This Row],[Limb_lodgment]]="FAIL",tblLoans[[#This Row],[Limb_b_rate]]="FAIL",tblLoans[[#This Row],[Limb_c_term]]="FAIL"),"NOT_COMPLYING",IF(OR(tblLoans[[#This Row],[Limb_a_written]]="UNKNOWN",tblLoans[[#This Row],[Limb_lodgment]]="UNKNOWN",tblLoans[[#This Row],[Limb_b_rate]]="UNKNOWN",tblLoans[[#This Row],[Limb_c_term]]="UNKNOWN"),"UNKNOWN","COMPLYING")))</f>
+        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[Floor_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"UNKNOWN",IF(OR(tblLoans[[#This Row],[Limb_a_written]]="FAIL",tblLoans[[#This Row],[Limb_lodgment]]="FAIL",tblLoans[[#This Row],[Limb_b_rate]]="FAIL",tblLoans[[#This Row],[Limb_c_term]]="FAIL"),"NOT_COMPLYING",IF(OR(tblLoans[[#This Row],[Limb_a_written]]="UNKNOWN",tblLoans[[#This Row],[Limb_lodgment]]="UNKNOWN",tblLoans[[#This Row],[Limb_b_rate]]="UNKNOWN",tblLoans[[#This Row],[Limb_c_term]]="UNKNOWN"),"UNKNOWN","COMPLYING"))))</f>
         <v/>
       </c>
       <c r="Y9" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(tblLoans[[#This Row],[Allowed_term_raw]]&lt;&gt;"",tblLoans[[#This Row],[Allowed_term_raw]],IF(AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),tblLoans[[#This Row],[maximum_term_years]]&lt;=7),7,"")))</f>
+        <f>IF(OR(tblLoans[[#This Row],[Status]]="SKIPPED",OR(LOWER(TRIM(tblLoans[[#This Row],[Floor_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),"",IF(tblLoans[[#This Row],[Allowed_term_raw]]&lt;&gt;"",tblLoans[[#This Row],[Allowed_term_raw]],IF(AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),tblLoans[[#This Row],[maximum_term_years]]&lt;=7),7,"")))</f>
         <v/>
       </c>
       <c r="Z9" s="9" t="str">
@@ -2253,11 +2328,11 @@
         <v/>
       </c>
       <c r="AB9" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")),TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")=Summary!$B$2,IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
+        <f>IF(tblLoans[[#This Row],[Status]]="SKIPPED","",IF(OR(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_made_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[Year_made_text]]),tblLoans[[#This Row],[Year_made_text]]=Summary!$B$2,IFERROR(VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&gt;Summary!$B$4,FALSE),AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),AND(ISNUMBER(Summary!$B$3),Summary!$B$3&lt;=0)),"REFUSED",IF(OR(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_made_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),NOT(ISNUMBER(Summary!$B$3)),NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),NOT(ISNUMBER(tblLoans[[#This Row],[Term_used]]))),"UNKNOWN",IF(tblLoans[[#This Row],[MYR_raw]]-ROUND(tblLoans[[#This Row],[payments_applied_during_the_year]],2)&lt;=0,"MYR_MET","MYR_SHORT"))))</f>
         <v/>
       </c>
       <c r="AC9" s="9" t="str">
-        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),"gate benchmark year differs from year_loan_made",IF(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;"")=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
+        <f>IF(tblLoans[[#This Row],[MYR_verdict]]="REFUSED",IF(tblLoans[[#This Row],[Gate_verdict]]&lt;&gt;"COMPLYING","s 109N gate is "&amp;tblLoans[[#This Row],[Gate_verdict]]&amp;", so s 109E produces no repayment figure",IF(tblLoans[[#This Row],[Floor_year]]&lt;&gt;tblLoans[[#This Row],[Year_made_text]],"gate benchmark year differs from year_loan_made",IF(tblLoans[[#This Row],[Year_made_text]]=Summary!$B$2,"year of income is the year the loan was made (s 109E(1)(a), s 109P)",IF(IFERROR(VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&gt;Summary!$B$4,FALSE),"loan made after the year of income",IF(AND(ISNUMBER(tblLoans[[#This Row],[Term_used]]),tblLoans[[#This Row],[Term_used]]&lt;=0),"nil remaining term under s 109E(6)","nil benchmark rate"))))),IF(tblLoans[[#This Row],[MYR_verdict]]="UNKNOWN",IF(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_made_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"}),"year_loan_made not established",IF(NOT(ISNUMBER(Summary!$B$3)),"no reviewed benchmark rate for the year of income",IF(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),"unpaid balance at end of previous year not established",IF(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),"payments applied not established","remaining term not established")))),""))</f>
         <v/>
       </c>
       <c r="AD9" s="10" t="str">
@@ -2281,12 +2356,20 @@
         <v>0</v>
       </c>
       <c r="AI9" s="9" t="str">
-        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""),4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))=7,MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),5,1)="-",ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),1,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),3,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),6,1))),ISNUMBER(VALUE(MID(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),7,1))),VALUE(RIGHT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),2))=MOD(VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))+1,100),VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&gt;=1900,VALUE(LEFT(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""),4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[payments_applied_during_the_year]]),N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</f>
+        <f>IF(TRIM(tblLoans[[#This Row],[out_of_scope_reason]]&amp;"")&lt;&gt;"","",TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_made_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[Year_made_text]])=7,MID(tblLoans[[#This Row],[Year_made_text]],5,1)="-",ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],1,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],2,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],3,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],4,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],6,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_made_text]],7,1))),VALUE(RIGHT(tblLoans[[#This Row],[Year_made_text]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))+1,100),VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&gt;=1900,VALUE(LEFT(tblLoans[[#This Row],[Year_made_text]],4))&lt;=2100),FALSE))),AND(tblLoans[[#This Row],[Status]]="REVIEWED",AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[Year_tested_text]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[Year_tested_text]])=7,MID(tblLoans[[#This Row],[Year_tested_text]],5,1)="-",ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],1,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],2,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],3,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],4,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],6,1))),ISNUMBER(VALUE(MID(tblLoans[[#This Row],[Year_tested_text]],7,1))),VALUE(RIGHT(tblLoans[[#This Row],[Year_tested_text]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[Year_tested_text]],4))+1,100),VALUE(LEFT(tblLoans[[#This Row],[Year_tested_text]],4))&gt;=1900,VALUE(LEFT(tblLoans[[#This Row],[Year_tested_text]],4))&lt;=2100),FALSE))))),"year label ","")&amp;IF(tblLoans[[#This Row],[Status]]&lt;&gt;"REVIEWED","",IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),N(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])&gt;1000000000000)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0,ROUND(N(tblLoans[[#This Row],[payments_applied_during_the_year]]),2)&lt;&gt;N(tblLoans[[#This Row],[payments_applied_during_the_year]]),N(tblLoans[[#This Row],[payments_applied_during_the_year]])&gt;1000000000000))))),"number ",""))))</f>
         <v/>
       </c>
       <c r="AJ9" s="9">
-        <f>IF(SUMPRODUCT((tblLoans[[#This Row],[loan_id]]&amp;""={"L-101","L-102","L-103","L-104","L-105","L-106","L-107","L-108"})*(tblLoans[[#This Row],[year_loan_made]]&amp;""={"2023-24","2022-23","2021-22","2024-25","2019-20","2020-21","2023-24","1996-97"}))&gt;0,1,0)</f>
+        <f>IF(SUMPRODUCT((tblLoans[[#This Row],[loan_id]]&amp;""={"L-101","L-102","L-103","L-104","L-105","L-106","L-107","L-108"})*(tblLoans[[#This Row],[Year_made_text]]&amp;""={"2023-24","2022-23","2021-22","2024-25","2019-20","2020-21","2023-24","1996-97"}))&gt;0,1,0)</f>
         <v>1</v>
+      </c>
+      <c r="AK9" s="9" t="str">
+        <f>TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(tblLoans[[#This Row],[year_loan_made]]&amp;"",_xlfn.UNICHAR(9)," "),_xlfn.UNICHAR(10)," "),_xlfn.UNICHAR(11)," "),_xlfn.UNICHAR(12)," "),_xlfn.UNICHAR(13)," "),_xlfn.UNICHAR(28)," "),_xlfn.UNICHAR(29)," "),_xlfn.UNICHAR(30)," "),_xlfn.UNICHAR(31)," "),_xlfn.UNICHAR(133)," "),_xlfn.UNICHAR(160)," "),_xlfn.UNICHAR(5760)," "),_xlfn.UNICHAR(8192)," "),_xlfn.UNICHAR(8193)," "),_xlfn.UNICHAR(8194)," "),_xlfn.UNICHAR(8195)," "),_xlfn.UNICHAR(8196)," "),_xlfn.UNICHAR(8197)," "),_xlfn.UNICHAR(8198)," "),_xlfn.UNICHAR(8199)," "),_xlfn.UNICHAR(8200)," "),_xlfn.UNICHAR(8201)," "),_xlfn.UNICHAR(8202)," "),_xlfn.UNICHAR(8232)," "),_xlfn.UNICHAR(8233)," "),_xlfn.UNICHAR(8239)," "),_xlfn.UNICHAR(8287)," "),_xlfn.UNICHAR(12288)," "))</f>
+        <v>1996-97</v>
+      </c>
+      <c r="AL9" s="9" t="str">
+        <f>TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;"",_xlfn.UNICHAR(9)," "),_xlfn.UNICHAR(10)," "),_xlfn.UNICHAR(11)," "),_xlfn.UNICHAR(12)," "),_xlfn.UNICHAR(13)," "),_xlfn.UNICHAR(28)," "),_xlfn.UNICHAR(29)," "),_xlfn.UNICHAR(30)," "),_xlfn.UNICHAR(31)," "),_xlfn.UNICHAR(133)," "),_xlfn.UNICHAR(160)," "),_xlfn.UNICHAR(5760)," "),_xlfn.UNICHAR(8192)," "),_xlfn.UNICHAR(8193)," "),_xlfn.UNICHAR(8194)," "),_xlfn.UNICHAR(8195)," "),_xlfn.UNICHAR(8196)," "),_xlfn.UNICHAR(8197)," "),_xlfn.UNICHAR(8198)," "),_xlfn.UNICHAR(8199)," "),_xlfn.UNICHAR(8200)," "),_xlfn.UNICHAR(8201)," "),_xlfn.UNICHAR(8202)," "),_xlfn.UNICHAR(8232)," "),_xlfn.UNICHAR(8233)," "),_xlfn.UNICHAR(8239)," "),_xlfn.UNICHAR(8287)," "),_xlfn.UNICHAR(12288)," "))</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -2312,214 +2395,214 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B2" s="7">
         <v>5.3699999999999998E-2</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B3" s="7">
         <v>4.5199999999999997E-2</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="F3" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="G3" s="7" t="s">
         <v>85</v>
-      </c>
-      <c r="G3" s="7" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B4" s="7">
         <v>4.5199999999999997E-2</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B5" s="7">
         <v>4.7699999999999999E-2</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B6" s="7">
         <v>8.2699999999999996E-2</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B7" s="7">
         <v>8.77E-2</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B8" s="7">
         <v>8.3699999999999997E-2</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B9" s="7">
         <v>8.77E-2</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -2541,21 +2624,21 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B1" s="5"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B3" s="12">
         <f>IFERROR(INDEX(tblRates[rate],MATCH(B2,tblRates[year_of_income],0)),"")</f>
@@ -2564,7 +2647,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B4" s="9">
         <f>IFERROR(VALUE(LEFT(B2,4)),"")</f>
@@ -2573,13 +2656,13 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B6" s="5"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B7" s="9">
         <f>COUNTIF(tblLoans[Status],"REVIEWED")</f>
@@ -2588,7 +2671,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B8" s="9">
         <f>COUNTIF(tblLoans[Gate_verdict],"COMPLYING")</f>
@@ -2597,7 +2680,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B9" s="9">
         <f>COUNTIF(tblLoans[Gate_verdict],"NOT_COMPLYING")</f>
@@ -2606,7 +2689,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B10" s="9">
         <f>COUNTIF(tblLoans[MYR_verdict],"MYR_MET")</f>
@@ -2615,7 +2698,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B11" s="9">
         <f>COUNTIF(tblLoans[MYR_verdict],"MYR_SHORT")</f>
@@ -2624,7 +2707,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B12" s="9">
         <f>SUM(tblLoans[Undecided])</f>
@@ -2633,7 +2716,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B13" s="9">
         <f>COUNTIF(tblLoans[MYR_verdict],"REFUSED")</f>
@@ -2642,7 +2725,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B14" s="9">
         <f>COUNTIF(tblLoans[Status],"SKIPPED")</f>
@@ -2651,7 +2734,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B15" s="10">
         <f>SUM(tblLoans[Exposure])</f>
@@ -2701,21 +2784,21 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B2" s="9" t="str">
         <f>IF(C2=0,"PASS","BLOCKED")</f>
@@ -2732,7 +2815,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B3" s="9" t="str">
         <f>IF(C3=0,"PASS","BLOCKED")</f>
@@ -2749,7 +2832,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B4" s="9" t="str">
         <f>IFERROR(IF(AND(ISNUMBER(Summary!B3),COUNT(tblRates[rate])=ROWS(tblRates[rate]),SUMPRODUCT(--(COUNTIF(tblRates[year_of_income],tblRates[year_of_income])&lt;&gt;1))=0,MIN(tblRates[rate])&gt;=0,MAX(tblRates[rate])&lt;=1),"PASS","BLOCKED"),"BLOCKED")</f>
@@ -2763,7 +2846,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B5" s="9" t="str">
         <f>IF(C5=0,"PASS","REVIEW")</f>
@@ -2780,7 +2863,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B6" s="9" t="str">
         <f>IF(C6=0,"PASS","REVIEW")</f>
@@ -2797,7 +2880,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B7" s="9" t="str">
         <f>IF(C7=0,"PASS","REVIEW")</f>
@@ -2814,7 +2897,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B8" s="9" t="str">
         <f>IF(C8=0,"PASS","REVIEW")</f>
@@ -2831,7 +2914,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B9" s="9" t="str">
         <f>IF(C9=0,"PASS","REVIEW")</f>
@@ -2857,32 +2940,32 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="135" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
   </sheetData>
@@ -2913,82 +2996,82 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B2" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B3" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B4" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B5" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B6" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B7" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B8" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B9" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B10" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Build the div7a workbook with the Rust builder and remove the Python one
The shipped workbook is regenerated through desktop Excel by the
build_workbook example. Against the committed workbook its model differs
only by the 2 accepted entries and the engine version (0.3.2 to 1.0.0);
every cached value equals the Excel-saved Python build's. The status
colours now display in Excel and each sheet names portrait A4.

The builder's formula tests move from the root tests/test_div7a_workbook.py
to builder.rs, which imports the engine constants they used to compare.
The Excel pass keeps the Python builder's force-disabled macros.
tests/test_shared_blocks.py drops the single-file Python group and pins
the Rust tooling copied from the payday builder.
</commit_message>
<xml_diff>
--- a/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
+++ b/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30527"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0A9D7CE-7C4F-4749-A564-608E431E2120}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ACFA53C-BE62-4172-8FC7-F9AAAE8BEC67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="-210" windowWidth="26010" windowHeight="21705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -65,7 +65,7 @@
     <t>Overall status</t>
   </si>
   <si>
-    <t>div7a-loan-review workbook, engine 0.3.2. Macro-free. Not advice; see DISCLAIMER.md in the repository.</t>
+    <t>div7a-loan-review workbook, engine 1.0.0. Macro-free. Not advice; see DISCLAIMER.md in the repository.</t>
   </si>
   <si>
     <t>loan_id</t>
@@ -455,7 +455,7 @@
     <t>Workbook engine version</t>
   </si>
   <si>
-    <t>0.3.2</t>
+    <t>1.0.0</t>
   </si>
   <si>
     <t>Desktop Excel build used to calculate cached values</t>
@@ -520,27 +520,37 @@
       <sz val="14"/>
       <color rgb="FF5C2D91"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="14"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF1F4E9E"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -553,16 +563,19 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF3F1F6"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF5C2D91"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE2E0DF"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -607,64 +620,64 @@
   <dxfs count="9">
     <dxf>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD4EDDA"/>
+        <patternFill>
+          <bgColor rgb="FFD4EDDA"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF3CD"/>
+        <patternFill>
+          <bgColor rgb="FFFFF3CD"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8D7DA"/>
+        <patternFill>
+          <bgColor rgb="FFF8D7DA"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD4EDDA"/>
+        <patternFill>
+          <bgColor rgb="FFD4EDDA"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF3CD"/>
+        <patternFill>
+          <bgColor rgb="FFFFF3CD"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8D7DA"/>
+        <patternFill>
+          <bgColor rgb="FFF8D7DA"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD4EDDA"/>
+        <patternFill>
+          <bgColor rgb="FFD4EDDA"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF3CD"/>
+        <patternFill>
+          <bgColor rgb="FFFFF3CD"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8D7DA"/>
+        <patternFill>
+          <bgColor rgb="FFF8D7DA"/>
         </patternFill>
       </fill>
     </dxf>
@@ -682,7 +695,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblLoans" displayName="tblLoans" ref="A1:AL9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblLoans" displayName="tblLoans" ref="A1:AL9" totalsRowShown="0">
   <tableColumns count="38">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="loan_id"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="borrower_reference"/>
@@ -776,7 +789,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="tblRates" displayName="tblRates" ref="A1:G9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="tblRates" displayName="tblRates" ref="A1:G9" totalsRowShown="0">
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="year_of_income"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="rate"/>
@@ -791,9 +804,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -831,7 +844,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -865,6 +878,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -899,9 +913,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1145,6 +1160,7 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="200" verticalDpi="200"/>
 </worksheet>
 </file>
 
@@ -2379,6 +2395,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="200" verticalDpi="200"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -2607,6 +2624,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="200" verticalDpi="200"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -2769,6 +2787,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="200" verticalDpi="200"/>
 </worksheet>
 </file>
 
@@ -2982,6 +3001,7 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="200" verticalDpi="200"/>
 </worksheet>
 </file>
 
@@ -3076,5 +3096,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="200" verticalDpi="200"/>
 </worksheet>
 </file>
</xml_diff>